<commit_message>
Rewrite batch 5 descriptions with sales-focused technical copy
Reemplaza las descripciones del lote 5 (237 productos) por una
versión que prioriza información técnica real (materiales, medidas,
capacidad, especificaciones) sobre frases vagas, corrige fichas
traducidas con redacción torpe y normaliza mayúsculas sueltas de
las fuentes originales.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bWxU7GBEhMMMrCBgBXSaR
</commit_message>
<xml_diff>
--- a/PRODUCTOS_RAPPI/ESTRUCTURA_RAPPI_LOTE5.xlsx
+++ b/PRODUCTOS_RAPPI/ESTRUCTURA_RAPPI_LOTE5.xlsx
@@ -614,10 +614,10 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>- Auriculares con funda de carga: auriculares inalámbricos para que no tengas que llevar esos auriculares con cable
-- La calidad de sonido estéreo de estos auriculares es excelente
-- También el emparejamiento es rápido
+- Ofrece sonido estéreo de alta calidad con emparejamiento rápido y estable
 - El auricular LED mostrará el estado de carga, y en la funda de carga inalámbrica, la pantalla digital LED inteligente puede comprobar la pantalla del consumo de batería en cualquier momento
-- Prácticos auriculares para llevar en tu bolsillo: la funda de carga es muy conveniente. No hay interrupciones al ver videos o jugar juegos</t>
+- Prácticos auriculares para llevar en tu bolsillo: su estuche de carga es compacto y práctico
+- Transmite audio sin cortes ni interrupciones al ver videos o jugar</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -642,11 +642,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>- DISPONIBLE EN COLOR NEGRO
-- Mouse inalámbrico recargable con conectividad Bluetooth 5.2 y receptor USB 2.4G para múltiples dispositivos
-- Diseño silencioso con clic izquierdo y derecho de bajo ruido para mayor comodidad en trabajo y estudio
+          <t>- Mouse inalámbrico recargable con conectividad Bluetooth 5.2 y receptor USB 2.4G para múltiples dispositivos
 - Iluminación LED RGB retroiluminada que aporta un estilo moderno y atractivo
-- Resolución ajustable de 800, 1200 y 1600 DPI para un control preciso según cada necesidad</t>
+- Resolución ajustable de 800, 1200 y 1600 DPI para un control preciso según cada necesidad
+- Batería de litio recargable integrada que elimina la necesidad de reemplazar pilas
+- Diseño compacto y ergonómico con dimensiones de 112 x 58 x 25 mm</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -671,11 +671,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>- DISPONIBLE EN COLOR NEGRO
-- Mouse inalámbrico recargable con conectividad Bluetooth 5.2 y receptor USB 2.4G para múltiples dispositivos
-- Diseño silencioso con clic izquierdo y derecho de bajo ruido para mayor comodidad en trabajo y estudio
+          <t>- Mouse inalámbrico recargable con conectividad Bluetooth 5.2 y receptor USB 2.4G para múltiples dispositivos
 - Iluminación LED RGB retroiluminada que aporta un estilo moderno y atractivo
-- Resolución ajustable de 800, 1200 y 1600 DPI para un control preciso según cada necesidad</t>
+- Resolución ajustable de 800, 1200 y 1600 DPI para un control preciso según cada necesidad
+- Batería de litio recargable integrada que elimina la necesidad de reemplazar pilas
+- Diseño compacto y ergonómico con dimensiones de 112 x 58 x 25 mm</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -703,8 +703,8 @@
           <t>- Herramienta compacta y práctica diseñada para cortar y pelar cables de forma rápida y precisa
 - Fabricado con acero, cromo, níquel y plástico para brindar resistencia y durabilidad
 - Medidas: Largo 15.2 cm x Ancho 12.7 cm
-- Cuenta con filo preciso para facilitar el pelado y corte de cables durante trabajos eléctricos
-- Incorpora un tope deslizante ajustable para facilitar el trabajo con diferentes cables</t>
+- Mango ergonómico antideslizante que proporciona comodidad y control durante el uso
+- Diseño de 5 pulgadas, práctico para trabajos que requieren precisión y facilidad de manejo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>- Difusor Humidificador Efecto Llama – Aromaterapia y Estilo
-- Transformá tus ambientes con un diseño innovador que combina humidificador y difusor de aromas en un solo producto
+          <t>- Difusor humidificador efecto llama – aromaterapia y estilo
 - Su efecto llama LED crea una atmósfera cálida y relajante, ideal para usar en el living, dormitorio, oficina o cualquier espacio de tu casa
-- Características principales
-- 2 en 1: Humidificador + difusor de aromaterapia</t>
+- 2 en 1: Humidificador + difusor de aromaterapia
+- Efecto llama LED: Iluminación que simula fuego real para un ambiente más acogedor
+- Fácil de usar: Carga por cable USB y controles simples</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -791,7 +791,7 @@
 - Incluye llaves hexagonales de diferentes tamaños: 1,5, 2, 2,5, 3, 4, 5, 6 y 8 mm, ofreciendo varias opciones para trabajar con distintos tipos de tornillos
 - Fabricadas en acero cromo vanadio con acabado satinado, estas llaves ofrecen una estructura resistente para el uso frecuente
 - Su diseño plegable permite guardar las llaves dentro del mango ergonómico, facilitando el almacenamiento y transporte del conjunto
-- Además, su formato compacto permite mantenerlas organizadas y listas para utilizar cuando las necesites</t>
+- El producto corresponde al modelo AM-I8855 y viene presentado en blíster</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -819,8 +819,8 @@
           <t>- Muñequera deportiva ideal para absorber el sudor durante el entrenamiento
 - Fabricada en 100% fibra sintética de poliéster
 - Medidas aproximadas: 8 x 8 cm
-- Presentación en par
-- Material super absorbente que ayuda a mantener el rostro seco</t>
+- Material super absorbente que ayuda a mantener el rostro seco
+- Con elástico cómodo que no incomoda ni aprieta durante la actividad física</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -932,11 +932,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>- Nombre: Panel LED 12W Sobreponer Luz Fresca
+          <t>- Nombre: panel LED 12w sobreponer luz fresca
 - Material: Aluminio de inyección para estabilidad de temperatura
 - Dimensiones: 17 cm x 17 cm - Potencia: 12W - Voltaje: 100-240V
 - Flujo luminoso: 1020 lm - Temperatura de color: 6500K (luz fría)
-- Ángulo de apertura: 120 grados - Índice de protección: IP20</t>
+- Fácil instalación, no requiere mantenimiento y alta durabilidad por su carcasa de aluminio de inyección</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -961,10 +961,10 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>- Panel LED Redondo Para Incrustar 12W Luz Blanca 6500K
+          <t>- Panel LED redondo para incrustar 12w luz blanca 6500k
 - Material: Aluminio y PMMA con difusor opalizado
 - Diámetro: 167 mm - Calado de incrustar: 126 mm
-- Potencia: 18W - Voltaje: 100-240V - Flujo luminoso: aprox. 780-960 lm
+- Potencia: 18W - Voltaje: 100-240V - Flujo luminoso: aprox
 - Temperatura de color: 6500K (luz blanca fría) - Ángulo de apertura: 120 grados</t>
         </is>
       </c>
@@ -1022,8 +1022,8 @@
           <t>- Medidas: 20 cm * 20 cm
 - Este producto es un Panel LED de la marca Macao (Modelo Incrustar/Sobreponer de 18W), diseñado para iluminación interior
 - Suele usarse en hogares o comercios, destacando por su alta eficiencia y ahorro energético
-- Características técnicas: Cuenta con una potencia de 18W y un driver integrado (el pequeño módulo blanco con cables) que regula la corriente eléctrica necesaria para que los LEDs funcionen de forma estable
-- Diseño: El diseño de la caja indica que sirve tanto para empotrar (incrustar) como para sobreponer, dependiendo del tipo de techo, con una certificación que avala su calidad</t>
+- Diseño: El diseño de la caja indica que sirve tanto para empotrar (incrustar) como para sobreponer, dependiendo del tipo de techo, con una certificación que avala su calidad
+- Instalación: Para instalarlo de manera segura en tu domicilio—o si necesitas repuestos y accesorios en tu área de Barranquilla—, puedes consultar tiendas locales de iluminación como Homecenter para encontrar productos similares</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1051,8 +1051,8 @@
           <t>- La línea de audífonos G-TIDE está diseñada para aquellos que valoran la durabilidad y la funcionalidad
 - Gracias a su micrófono incorporado, podrás atender tus llamadas con facilidad, asegurando que no te pierdas de ninguna conversación importante
 - Este modelo es especialmente apreciado por los gamers, que encuentran en él una herramienta efectiva para comunicarse y sumergirse en su experiencia de juego
-- Características:
-- Sonido Digital Superior</t>
+- Compatibles con Smartphones
+- Durabilidad y Funcionalidad</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1081,7 +1081,7 @@
 - Incluye: cepillo de cerdas suaves, peine de puntas redondeadas, tijera de punta segura, cortauñas, lima y adaptador
 - Fabricado en material ABS resistente, libre de BPA y no tóxico
 - Cerdas delicadas ideales para el cuero cabelludo sensible del recién nacido
-- Tijera con punta redondeada para mayor seguridad al cortar uñas</t>
+- Producto ligero (200 g), práctico para llevar en la pañalera o bolso maternal</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1110,7 +1110,7 @@
 - Incluye: cepillo de cerdas suaves, peine de puntas redondeadas, tijera de punta segura, cortauñas, lima y adaptador
 - Fabricado en material ABS resistente, libre de BPA y no tóxico
 - Cerdas delicadas ideales para el cuero cabelludo sensible del recién nacido
-- Tijera con punta redondeada para mayor seguridad al cortar uñas</t>
+- Producto ligero (200 g), práctico para llevar en la pañalera o bolso maternal</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1139,7 +1139,7 @@
 - Incluye: cepillo de cerdas suaves, peine de puntas redondeadas, tijera de punta segura, cortauñas, lima y adaptador
 - Fabricado en material ABS resistente, libre de BPA y no tóxico
 - Cerdas delicadas ideales para el cuero cabelludo sensible del recién nacido
-- Tijera con punta redondeada para mayor seguridad al cortar uñas</t>
+- Producto ligero (200 g), práctico para llevar en la pañalera o bolso maternal</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1193,11 +1193,11 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>- Características principales:
-- Linterna LED potente integrada: Luz ubicada en la base del mango para brindar visibilidad nocturna y evitar charcos o tropiezos en la calle
+          <t>- Linterna LED potente integrada: Luz ubicada en la base del mango para brindar visibilidad nocturna y evitar charcos o tropiezos en la calle
 - Apertura y cierre automático: Botón intuitivo que despliega y recoge la sombrilla rápidamente con una sola mano
 - Protección solar y lluvia: Tela de alta densidad repelente al agua y equipada con filtro de protección contra rayos UV
-- Estructura robusta antiviento: Varillas flexibles y resistentes diseñadas para soportar ráfagas de viento sin deformarse</t>
+- Estructura robusta antiviento: Varillas flexibles y resistentes diseñadas para soportar ráfagas de viento sin deformarse
+- Mango ergonómico en tono negro mate: Empuñadura suave al tacto con refinado bisel metálico cromado</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1222,11 +1222,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>- Características principales:
-- Linterna LED potente integrada: Luz ubicada en la base del mango para brindar visibilidad nocturna y evitar charcos o tropiezos en la calle
+          <t>- Linterna LED potente integrada: Luz ubicada en la base del mango para brindar visibilidad nocturna y evitar charcos o tropiezos en la calle
 - Apertura y cierre automático: Botón intuitivo que despliega y recoge la sombrilla rápidamente con una sola mano
 - Protección solar y lluvia: Tela de alta densidad repelente al agua y equipada con filtro de protección contra rayos UV
-- Estructura robusta antiviento: Varillas flexibles y resistentes diseñadas para soportar ráfagas de viento sin deformarse</t>
+- Estructura robusta antiviento: Varillas flexibles y resistentes diseñadas para soportar ráfagas de viento sin deformarse
+- Mango ergonómico en tono azul claro mate: Empuñadura suave al tacto con refinado bisel metálico cromado</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1251,11 +1251,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>- Características principales:
-- Linterna LED potente integrada: Luz ubicada en la base del mango para brindar visibilidad nocturna y evitar charcos o tropiezos en la calle
+          <t>- Linterna LED potente integrada: Luz ubicada en la base del mango para brindar visibilidad nocturna y evitar charcos o tropiezos en la calle
 - Apertura y cierre automático: Botón intuitivo que despliega y recoge la sombrilla rápidamente con una sola mano
 - Protección solar y lluvia: Tela de alta densidad repelente al agua y equipada con filtro de protección contra rayos UV
-- Estructura robusta antiviento: Varillas flexibles y resistentes diseñadas para soportar ráfagas de viento sin deformarse</t>
+- Estructura robusta antiviento: Varillas flexibles y resistentes diseñadas para soportar ráfagas de viento sin deformarse
+- Mango ergonómico en tono azul oscuro mate: Empuñadura suave al tacto con refinado bisel metálico cromado</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1280,11 +1280,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>- Características principales:
-- Linterna LED potente integrada: Luz ubicada en la base del mango para brindar visibilidad nocturna y evitar charcos o tropiezos en la calle
+          <t>- Linterna LED potente integrada: Luz ubicada en la base del mango para brindar visibilidad nocturna y evitar charcos o tropiezos en la calle
 - Apertura y cierre automático: Botón intuitivo que despliega y recoge la sombrilla rápidamente con una sola mano
 - Protección solar y lluvia: Tela de alta densidad repelente al agua y equipada con filtro de protección contra rayos UV
-- Estructura robusta antiviento: Varillas flexibles y resistentes diseñadas para soportar ráfagas de viento sin deformarse</t>
+- Estructura robusta antiviento: Varillas flexibles y resistentes diseñadas para soportar ráfagas de viento sin deformarse
+- Mango ergonómico en tono rojo mate: Empuñadura suave al tacto con refinado bisel metálico cromado</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1309,11 +1309,11 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>- Características principales:
-- Linterna LED potente integrada: Luz ubicada en la base del mango para brindar visibilidad nocturna y evitar charcos o tropiezos en la calle
+          <t>- Linterna LED potente integrada: Luz ubicada en la base del mango para brindar visibilidad nocturna y evitar charcos o tropiezos en la calle
 - Apertura y cierre automático: Botón intuitivo que despliega y recoge la sombrilla rápidamente con una sola mano
 - Protección solar y lluvia: Tela de alta densidad repelente al agua y equipada con filtro de protección contra rayos UV
-- Estructura robusta antiviento: Varillas flexibles y resistentes diseñadas para soportar ráfagas de viento sin deformarse</t>
+- Estructura robusta antiviento: Varillas flexibles y resistentes diseñadas para soportar ráfagas de viento sin deformarse
+- Mango ergonómico en tono verde mate: Empuñadura suave al tacto con refinado bisel metálico cromado</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1339,10 +1339,10 @@
       <c r="C30" t="inlineStr">
         <is>
           <t>- — Nombre: Grifo Giratorio 3 en 1 con 360 grados — Modelo: HY-035
-- — Material: Acero inoxidable — Válvula: CPVC
-- — Rotación de 360 grados — 3 funciones en un solo grifo. 14CM X 3.7CM
+- — material: acero inoxidable — válvula: cpvc
+- — Rotación de 360 grados — 3 funciones en un solo grifo
 - — Rotación completa de 360° que permite dirigir el flujo de agua en cualquier dirección con total facilidad
-- — Sistema 3 en 1 que combina múltiples modos de salida de agua en un solo accesorio</t>
+- — Fabricado en acero inoxidable de alta resistencia con válvula CPVC para mayor durabilidad y resistencia a la corrosión</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1367,11 +1367,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>- Diámetro: 26 cm, tamaño adecuado para mascotas pequeñas y medianas. 24 onzas
+          <t>- Diámetro: 26 cm, tamaño adecuado para mascotas pequeñas y medianas
 - Fabricado en metal de acabado metálico plateado, con material libre de BPA y PVC y diseño no tóxico
 - Ideal para servir alimentos y agua a perros y gatos durante su rutina diaria
 - Diseño robusto, práctico y fácil de limpiar, pensado para soportar el uso cotidiano
-- Tipo de alimentación manual, sin sistema automático ni diseño plegable</t>
+- Contenido: 1 plato comedero metálico para mascotas</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1590,7 +1590,8 @@
         <is>
           <t>- Diadema de spa para mujer con forro de esponja y tela de rizo que cubre la superficie
 - Estas diademas para el cuidado de la piel tienen una fuerte función de absorción de agua y se pueden usar cuando te lavas la cara, te cuidas la piel o te maquillas
-- Las pulseras están hechas de vellón coralino de calidad. Y las pulseras también tienen buena elasticidad y se pueden estirar para adaptarse mejor a su muñeca</t>
+- Las pulseras están hechas de vellón coralino de calidad
+- Y las pulseras también tienen buena elasticidad y se pueden estirar para adaptarse mejor a su muñeca</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1753,9 +1754,9 @@
         <is>
           <t>- Ilumina tus celebraciones con el Bombillo Proyector Navideño LED Multifigura con Adaptador, diseñado para crear ambientes llenos de color y espíritu festivo
 - Su tecnología LED proyecta figuras navideñas y patrones multicolores en movimiento, convirtiendo paredes y espacios interiores en una decoración llamativa
-- Cuenta con rosca E27 convencional y puede utilizarse en portalámparas o directamente en una toma de corriente gracias al adaptador incluido
-- Su diseño reflector giratorio permite disfrutar de una proyección dinámica de figuras como estrellas, muñecos de nieve y diferentes patrones de colores
-- Es ideal para decorar salas, dormitorios, comedores, vitrinas, locales, oficinas y espacios para eventos, así como para Navidad, reuniones familiares, cenas y otras celebraciones</t>
+- Su instalación es sencilla: solo debes colocar el bombillo en el adaptador y conectarlo a una toma de 110 V, o instalarlo en un casquillo E27 convencional
+- Fabricado en plástico ABS, tiene unas dimensiones aproximadas de 13 cm de alto por 6,5 cm de ancho y un peso de 95 g
+- Su tecnología LED</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1784,7 +1785,7 @@
 - Su tecnología LED de bajo consumo proyecta figuras navideñas en movimiento, como muñecos de nieve, estrellas y patrones multicolores
 - Además, su diseño versátil permite utilizarlo en un portalámparas convencional o directamente en una toma de corriente gracias al adaptador incluido
 - Es ideal para decorar salas, dormitorios, comedores, oficinas, locales, vitrinas y espacios para eventos especiales
-- Su proyección giratoria crea un ambiente acogedor y llamativo para Navidad, reuniones familiares, cenas, celebraciones de Nochebuena y otras ocasiones</t>
+- Para utilizarlo directamente en una toma, solo debes insertar el bombillo en el adaptador incluido y conectarlo a una toma de corriente de 110 V; si deseas usarlo en una lámpara, puedes enroscarlo en un casquillo convencional</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1810,8 +1811,10 @@
       <c r="C47" t="inlineStr">
         <is>
           <t>- Se puede usar para liberar dolor e incomodidad inmediatamente en cualquier lugar y en cualquier momento
-- Utiliza rodillo de hielo para eliminar la fatiga ocular. Rodillo instantáneo para aliviar el dolor en cualquier parte de tu cuerpo
-- Las heridas leves, las quemaduras y las picaduras de insectos pueden usar rodillos de hielo. Después del afeitado, calma y calma su piel con un rodillo de hielo</t>
+- Utiliza rodillo de hielo para eliminar la fatiga ocular
+- Rodillo instantáneo para aliviar el dolor en cualquier parte de tu cuerpo
+- Las heridas leves, las quemaduras y las picaduras de insectos pueden usar rodillos de hielo
+- Después del afeitado, calma y calma su piel con un rodillo de hielo</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1977,9 +1980,9 @@
         <is>
           <t>- Esta preciosa bolsa térmica grande, es perfecta para calentar tus manos o piernas durante los días fríos, para aliviar los dolorosos cólicos menstruales o los dolores musculares provocados por algún esfuerzo físico
 - Su capacidad es de 500 ML
-- Solo debes calentar un poco de agua, llenar la bolsa y disfrutar de la suave sensación del calor junto al material de peluche/felpa del forro de la misma, además este forro es el encargado de mantener caliente el agua por mucho más tiempo
 - Alivio del dolor: El calor ayuda a dilatar los vasos sanguíneos y mejora la circulación, lo que puede reducir el dolor
-- Relajación muscular: Ayuda a relajar los músculos tensos y reduce los espasmos.Confort: Proporciona una sensación de confort y bienestar durante el uso</t>
+- Relajación muscular: Ayuda a relajar los músculos tensos y reduce los espasmos.Confort: Proporciona una sensación de confort y bienestar durante el uso
+- Botella de agua caliente cómoda y cálida con tapón roscado grande, costura y boca impermeable, sellada y a prueba de fugas, capacidad súper grande de 500 ml, se recomienda llenar dos tercios</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2004,11 +2007,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>- Disfruta de un momento de relajación en casa o durante tus viajes con esta Almohada de Masaje Shiatsu, diseñada con un formato delgado, ligero y ergonómico que se adapta cómodamente a diferentes zonas del cuerpo
-- Incorpora cuatro cabezales de masaje con rodillos duales y cuatro nodos que realizan un movimiento de amasamiento profundo, ideal para ayudar a relajar los músculos y disminuir la sensación de tensión en cuello, espalda, cintura, cadera, piernas, pantorrillas y muslos
-- Su función de calor incorporado proporciona una sensación cálida y relajante que complementa el masaje, ayudando a relajar la zona tratada
-- Puedes activar o desactivar el calor de manera independiente, mientras que su sistema de protección contra sobrecalentamiento incluye apagado automático después de un periodo de funcionamiento continuo
-- Para un uso adecuado, se recomienda utilizarla durante aproximadamente 15 minutos por sesión y mantenerla alejada del agua, la humedad y fuentes de fuego</t>
+          <t>- Su función de calor incorporado proporciona una sensación cálida y relajante que complementa el masaje, ayudando a relajar la zona tratada
+- Para un uso adecuado, se recomienda utilizarla durante aproximadamente 15 minutos por sesión y mantenerla alejada del agua, la humedad y fuentes de fuego
+- Fabricada en cuero sintético PU, tela y componentes mecánicos, cuenta con una banda elástica integrada que permite fijarla al respaldo de una silla, convirtiéndola en una opción práctica para utilizar en el automóvil
+- Incluye adaptador para auto de 12V y adaptador de corriente AC de 220V/50Hz y 20W
+- Su tamaño aproximado es de 30 x 18 x 9 cm y su peso es de 992 g, ofreciendo una solución compacta y versátil para disfrutar de masajes relajantes donde lo necesites</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2037,7 +2040,7 @@
 - Con unas medidas de 65 x 35 cm, esta alfombra es perfecta para bañeras y entradas de baño, brindando un toque moderno y ambiental a tu espacio
 - Su diseño antideslizante garantiza una experiencia segura, evitando resbalones y caídas
 - Fabricada en 100% PVC, este material no solo es duradero, sino que también es fácil de limpiar
-- Aunque no es absorbente, su superficie permite un secado rápido. La alfombra es nueva y pertenece a la línea TRANSPARENTE, lo que la convierte en una elección elegante y funcional</t>
+- Aunque no es absorbente, su superficie permite un secado rápido</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2066,7 +2069,7 @@
 - Con unas medidas de 65 x 35 cm, esta alfombra es perfecta para bañeras y entradas de baño, brindando un toque moderno y ambiental a tu espacio
 - Su diseño antideslizante garantiza una experiencia segura, evitando resbalones y caídas
 - Fabricada en 100% PVC, este material no solo es duradero, sino que también es fácil de limpiar
-- Aunque no es absorbente, su superficie permite un secado rápido. La alfombra es nueva y pertenece a la línea TRANSPARENTE, lo que la convierte en una elección elegante y funcional</t>
+- Aunque no es absorbente, su superficie permite un secado rápido</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2095,7 +2098,7 @@
 - Con unas medidas de 65 x 35 cm, esta alfombra es perfecta para bañeras y entradas de baño, brindando un toque moderno y ambiental a tu espacio
 - Su diseño antideslizante garantiza una experiencia segura, evitando resbalones y caídas
 - Fabricada en 100% PVC, este material no solo es duradero, sino que también es fácil de limpiar
-- Aunque no es absorbente, su superficie permite un secado rápido. La alfombra es nueva y pertenece a la línea TRANSPARENTE, lo que la convierte en una elección elegante y funcional</t>
+- Aunque no es absorbente, su superficie permite un secado rápido</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2150,10 +2153,10 @@
       <c r="C59" t="inlineStr">
         <is>
           <t>- Mantén tus utensilios de cocina siempre organizados y al alcance con este cubiertero giratorio
-- Su diseño moderno y funcional en acabado metálico te permite acceder fácilmente a cada compartimiento gracias a su base giratoria, ideal para optimizar espacios en la cocina o el comedor, dándote la comodidad de tener todo a la mano y listo para usar en tu día a día
 - Disfruta de la comodidad de tener tus cubiertos siempre a la vista y de fácil acceso gracias a su diseño totalmente ensamblado y giratorio
 - Optimiza el espacio en tu cocina con un porta utensilios que mide 18 cm de alto, brindando una solución compacta y eficiente
-- Añade un toque moderno y elegante a tu hogar con el acabado metálico de este organizador, ideal para cualquier estilo de decoración</t>
+- Añade un toque moderno y elegante a tu hogar con el acabado metálico de este organizador, ideal para cualquier estilo de decoración
+- Aprovecha su funcionalidad para almacenar diversos utensilios de uso diario, manteniendo tu cocina ordenada con capacidad para dos elementos</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2182,7 +2185,7 @@
 - Este contenedor multiusos combina a la perfección la elegancia visual del tejido tipo rattan con la máxima durabilidad del plástico de alta densidad
 - Su diseño compacto y estilizado la convierte en el accesorio de almacenamiento ideal para mantener cada rincón de tu hogar perfectamente impecable y libre de desorden
 - Acabado calado transpirable: Paredes perforadas con patrón de rattan que permiten una excelente ventilación, evitando la acumulación de humedad y malos olores
-- Asas integradas: Laterales diseñados con ranuras ergonómicas para un agarre cómodo y un transporte seguro entre habitaciones</t>
+- Fácil de limpiar: Superficie plástica impermeable que se lava de forma rápida con agua o se limpia pasando simplemente un paño húmedo</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2323,9 +2326,9 @@
       <c r="C65" t="inlineStr">
         <is>
           <t>- Limpiavidrios Magnético ofrece eficiencia y seguridad, asegurando que tus ventanas queden impecables desde el interior y exterior, sin esfuerzo ni riesgos
-- ESPECIFICACIONES:
-- Material: ABS, Látex natural, Imán NdFeB
-- Diseño triangular completo Cuerda de Seguridad: 2 metros de longitud. Efectivo para ventanas de doble acristalamiento de 15-24 mm de espesor</t>
+- Material: ABS, látex natural, imán ndfeb
+- Diseño triangular completo Cuerda de Seguridad: 2 metros de longitud
+- Efectivo para ventanas de doble acristalamiento de 15-24 mm de espesor</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2354,7 +2357,7 @@
 - Material antiadherente y flexible que permite desmoldar fácilmente los alimentos y garantiza una cocción uniforme
 - Alta resistencia al calor, soporta temperaturas aproximadas entre -40 °C y 230–240 °C, ideal para múltiples preparaciones
 - Apto para freidora de aire, horno, microondas, sartén y otros electrodomésticos de cocina
-- Diseño práctico con asas laterales que facilitan el agarre y la manipulación segura del molde</t>
+- Tamaño aproximado de 8.1 x 8.1 x 2.1 pulgadas, compatible con la mayoría de las freidoras de aire</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2379,7 +2382,10 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>- Adhesivo reutilizable. Resistente al agua. Transparente. No deja residuos. Soporta hasta 1 kg</t>
+          <t>- Adhesivo reutilizable
+- Resistente al agua
+- No deja residuos
+- Soporta hasta 1 kg</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2429,11 +2435,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>- Completamente automático
-- Diámetro abierto :100cm
+          <t>- Diámetro abierto :100cm
 - Estilo de diseño : Contemporáneo
 - Grupo de edad : Adultos y Niños
-- Material de los paneles : Pongis</t>
+- Material de los paneles : Pongis
+- Material : Tela de nailon 190T</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2460,7 +2466,7 @@
         <is>
           <t>- CHAQUETA: 63cm de ancho x 75 cm de largo
 - PANTALON: 100cm de largo
-- Este impermeable no es solo un uniforme, es un escudo contra los elementos:
+- Este impermeable no es solo un uniforme, es un escudo contra los elementos
 - Material impermeable: Te mantiene completamente seco, incluso en los días más lluviosos
 - Excelente calidad: Diseñado para resistir el uso intensivo y las condiciones climáticas más exigentes</t>
         </is>
@@ -2489,7 +2495,7 @@
         <is>
           <t>- CHAQUETA: 66cm de ancho x 80 cm de largo
 - PANTALON: 103cm de largo
-- Este impermeable no es solo un uniforme, es un escudo contra los elementos:
+- Este impermeable no es solo un uniforme, es un escudo contra los elementos
 - Material impermeable: Te mantiene completamente seco, incluso en los días más lluviosos
 - Excelente calidad: Diseñado para resistir el uso intensivo y las condiciones climáticas más exigentes</t>
         </is>
@@ -2660,8 +2666,8 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>- No solo es hermoso, sino también práctico. Parece Mármol Real, que puede satisfacer la visión sin parecer artificial
-- Estos papeles tipo Mármol son suaves e insonorizados, brillantes, hermosos y adecuados para la zona de juego de los niños, desempeñando una función leve de papel de anticolisión y aislamiento acústico, proporcionando un espacio seguro y silencioso para ti y tu familia
+          <t>- No solo es hermoso, sino también práctico
+- Parece Mármol Real, que puede satisfacer la visión sin parecer artificial
 - Dimensiones: 60 cm x 30 cm por lámina
 - Resistencia: Impermeable y resistente al aceite (ideal para salpicaderos de cocina o baños)
 - Superficies Aptas: Baldosa, madera, metal, vidrio o paredes lisas pintadas</t>
@@ -2689,8 +2695,8 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>- No solo es hermoso, sino también práctico. Parece Mármol Real, que puede satisfacer la visión sin parecer artificial
-- Estos papeles tipo Mármol son suaves e insonorizados, brillantes, hermosos y adecuados para la zona de juego de los niños, desempeñando una función leve de papel de anticolisión y aislamiento acústico, proporcionando un espacio seguro y silencioso para ti y tu familia
+          <t>- No solo es hermoso, sino también práctico
+- Parece Mármol Real, que puede satisfacer la visión sin parecer artificial
 - Dimensiones: 60 cm x 30 cm por lámina
 - Resistencia: Impermeable y resistente al aceite (ideal para salpicaderos de cocina o baños)
 - Superficies Aptas: Baldosa, madera, metal, vidrio o paredes lisas pintadas</t>
@@ -2721,8 +2727,8 @@
           <t>- Maximiza la eficiencia y la organización en tu cocina con el Posillero de 60 cm
 - Este versátil accesorio está diseñado para su uso en muebles altos y está fabricado en acero plastificado, asegurando durabilidad y resistencia a la corrosión
 - Portavasos, pocillero, platera, rejilla escurridora en acero plastificado
-- Fabricado en acero con recubrimiento plastificado de alta resistencia, este accesorio es la solución ideal para la organización de vajilla en cocinas que buscan durabilidad y una excelente relación costo-beneficio
-- Se adapta a módulos de 600 mm, ofreciendo una protección superior contra la corrosión y la humedad propia de la zona del fregadero</t>
+- Se adapta a módulos de 600 mm, ofreciendo una protección superior contra la corrosión y la humedad propia de la zona del fregadero
+- Su diseño optimizado permite un almacenamiento seguro y ordenado de vasos y pocillos, maximizando el espacio interno de los gabinetes superiores</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2747,11 +2753,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>- destornillador para reparaciones de emergencia, equipado con una variedad de diferentes cuchillas, que soportan la mayoría de los tornillos
+          <t>- Destornillador para reparaciones de emergencia, equipado con una variedad de diferentes cuchillas, que soportan la mayoría de los tornillos
 - Imprescindible para ciclistas nuevos y experimentados
-- Caracteristicas:
 - Linterna integrada para uso por sí sola o para iluminar
-- Cabezas magnéticas de aleación de acero CRV</t>
+- 6 LED de gran alcance
+- Tamaño: 12,6*4,8*5cm</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2776,7 +2782,9 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>- MINI MOUSE ÓPTICO -INTERFAZ: USB 2.0 -3 BOTONES -DPI 1000 -COLOR: NEGRO -CABLE: 1,25 M -LUZ ROJA -PLUG&amp;PLAY -SCROLL -TAMAÑO 96*52*34 -COMPATIBLE CON: WINDOWS, MAC OS 10,5 Y LINUX</t>
+          <t>- MINI MOUSE ÓPTICO
+- Interfaz: USB 2.0 -3 botones
+- Compatible con: windows, mac os 10,5 y linux</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2804,8 +2812,8 @@
           <t>- Medidas aproximadas: 10.5 cm de largo x 5.5 cm de ancho x 2.5 cm de alto; peso de 99 g
 - Fabricado con polímero de alta resistencia, diseñado para ofrecer durabilidad y un manejo cómodo
 - Dispositivo de defensa personal con linterna LED integrada para facilitar la visibilidad en condiciones de poca iluminación
-- Diseño compacto y portátil que permite transportarlo fácilmente en bolsillos, bolsos o compartimentos pequeños
-- Batería recargable mediante cargador incluido para un uso práctico y continuo</t>
+- Batería recargable mediante cargador incluido para un uso práctico y continuo
+- Contenido del paquete: 1 dispositivo modelo VTR-206, 1 cargador y 1 funda de transporte</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2888,11 +2896,11 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>- Nuevo Kit de Caligrafía para Niños: Aprendizaje Divertido y Mágico a tu Alcance, cuaderno de caligrafía en inglés, para que tus niños aprendan nuevos idiomas desde pequeños
-- Presentamos el kit de caligrafía definitivo que hará que aprender sea una aventura para tus pequeños
-- Este set exclusivo incluye cuatro libros interactivos diseñados meticulosamente para fomentar el desarrollo de habilidades esenciales en matemáticas, dibujo, alfabetización y numeración de manera divertida y estimulante
-- Los niños aprenden por repetición y con estos LIBROS MAGICOS podrán rellenar una y otra vez los libros gracias a la tinta innovadora. LA TINTA DESAPARECE EN MINUTOS
-- ¿Qué Incluye el Kit? - 1 Libro de Matemáticas: Juegos y actividades para enamorarse de los números</t>
+          <t>- ¿Qué Incluye el Kit? - 1 Libro de Matemáticas: Juegos y actividades para enamorarse de los números
+- - 1 Libro de Dibujo: Expresa tu creatividad con cada trazo
+- - 1 Libro del Alfabeto: Aventuras de A a Z para maestros de la caligrafía en potencia
+- - 1 Libro de Números: Diversión contando, sumando y restando
+- Medida 19 cm x 13 cm</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2917,11 +2925,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>- ALMOHADA PARA PIERNAS Y APOYO DE RODILLAS ERGONÓMICA LEG PILLOW CON OUR
+          <t>- Almohada para piernas y apoyo de rodillas ergonómica leg pillow con our
 - Además, la almohada está ventilada, lo que promueve el flujo de aire durante toda la noche y te mantiene fresco durante toda la noche
-- CARACTERÍSTICAS:
 - * Ayuda a restaurar tu alineación natural
-- * Reduce la presión en las rodillas, las caderas y la parte baja de la espalda</t>
+- * Medidas: 25 cm x 13 cm x 23 cm
+- *Material: Espuma de poliuretano</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2948,9 +2956,9 @@
         <is>
           <t>- Organiza tu equipaje de forma práctica con este Set de 6 Piezas Organizadoras de Viaje, diseñado para mantener tus pertenencias ordenadas y aprovechar mejor el espacio al empacar
 - Sus diferentes tamaños permiten separar ropa, maquillaje, zapatos y otros artículos de manera sencilla, evitando el desorden dentro de la maleta
-- Es una opción práctica para viajes, vacaciones o escapadas
 - Las bolsas están fabricadas en poliéster resistente al agua y cuentan con un diseño de malla que favorece la ventilación, además de ayudar a proteger tus pertenencias de la humedad
-- El set está disponible en colores negro, vino tinto, gris, sandía, rosa, azul y celeste, sujetos a disponibilidad</t>
+- Las bolsas de malla tienen medidas aproximadas de 37 x 27 x 12 cm, 30 x 20 x 12 cm y 20 x 15 x 12 cm en sus tamaños grande, mediano y pequeño
+- Las bolsas completas miden aproximadamente 31 x 23 cm, 26 x 19 cm y 17 x 13 cm respectivamente</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2976,8 +2984,7 @@
       <c r="C88" t="inlineStr">
         <is>
           <t>- El bloqueo funciona bloqueando la palanca del freno delantero en el manillar para evitar que el vehículo se aleje, la solución perfecta para el estacionamiento a corto plazo
-- Material: plástico ABS
-- Esta Cerradura Antirrobo Es Muy Resistente Y A Prueba De Manipulaciones Puede Prevenir Eficazmente El Robo De Motocicletas</t>
+- Esta cerradura antirrobo es muy resistente y a prueba de manipulaciones puede prevenir eficazmente el robo de motocicletas</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -3002,8 +3009,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>- Material: Plástico
-- Material impermeable, la cubierta superior de la bicicleta está hecha de plástico, nailon y fibra de PVC
+          <t>- Material impermeable, la cubierta superior de la bicicleta está hecha de plástico, nailon y fibra de PVC
 - Este soporte para teléfono tiene una cabeza de bola giratoria de rotación de 360 grados, su brazo se puede girar hacia arriba y hacia abajo, te permite girar libremente la pantalla de tu teléfono según cualquier orientación que se adapte a tus preferencias</t>
         </is>
       </c>
@@ -3031,9 +3037,9 @@
         <is>
           <t>- Este genial juego de memoria te ofrece una gran variedad de juegos con los que poner a prueba tus reflejos, memoria y más
 - Un juguete con el tamaño ideal para llevarlo a todas partes y fabricado con materiales de gran calidad y resistencia
-- Escoge tu juego preferido y acepta el reto más genial, pon a prueba tus reflejos con Golpea a Topo, mejora tu memoria con el juego específico para ello y descubre tus habilidades rítmicas con el Maestro del Ritmo y Toca el Piano
-- Edad recomendada. 3 años o más
-- Incluye: 1 juego electrónico de memoria 4 en 1 con luz, sonidos y varios estilos de juego</t>
+- Incluye: 1 juego electrónico de memoria 4 en 1 con luz, sonidos y varios estilos de juego
+- Medidas aproximadas del juguete: 2,5 cm de alto, 13 cm de ancho y 13,5 cm de fondo
+- Funciona con 2 pilas "AAA"</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -3062,7 +3068,7 @@
 - Estos individuales de encaje bordado con diseño europeo añaden un toque de sofisticación clásica a cualquier cena
 - El equilibrio perfecto entre arte y funcionalidad para recibir a tus invitados con distinción
 - Técnica: Bordado a máquina de alta precisión con acabado calado, lo que permite ver la superficie de la mesa a través de los patrones de encaje
-- Estampado: Motivos florales y arabescos clásicos. Forma: Rectangular con bordes festoneados (u ondulados) siguiendo la forma del encaje</t>
+- Estampado: Motivos florales y arabescos clásicos</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3169,8 +3175,8 @@
           <t>- Trituradora de pollo mejorada Krafty con dientes más largos y afilados, mango ergonómico cómodo y tapa transparente que permite visualizar fácilmente el proceso de trituración
 - Sistema de trituración rápida y uniforme con dientes de plástico de doble nivel y puntas en la tapa que sujetan la carne de forma segura para resultados consistentes
 - Ideal para desmenuzar pollo, cerdo, res y verduras, perfecta para tacos, ensaladas, sándwiches, enchiladas, quesadillas, cazuelas, comidas fitness y comida para mascotas
-- Fabricada con materiales de alta calidad, libres de BPA y certificados por la FDA, segura para uso diario y altamente duradera
-- Diseño antideslizante con base de goma en forma de flor que brinda mayor estabilidad, seguridad y comodidad durante el uso</t>
+- Diseño antideslizante con base de goma en forma de flor que brinda mayor estabilidad, seguridad y comodidad durante el uso
+- Tamaño: 19x19x7 cm</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -3198,8 +3204,8 @@
           <t>- Trituradora de pollo mejorada Krafty con dientes más largos y afilados, mango ergonómico cómodo y tapa transparente que permite visualizar fácilmente el proceso de trituración
 - Sistema de trituración rápida y uniforme con dientes de plástico de doble nivel y puntas en la tapa que sujetan la carne de forma segura para resultados consistentes
 - Ideal para desmenuzar pollo, cerdo, res y verduras, perfecta para tacos, ensaladas, sándwiches, enchiladas, quesadillas, cazuelas, comidas fitness y comida para mascotas
-- Fabricada con materiales de alta calidad, libres de BPA y certificados por la FDA, segura para uso diario y altamente duradera
-- Diseño antideslizante con base de goma en forma de flor que brinda mayor estabilidad, seguridad y comodidad durante el uso</t>
+- Diseño antideslizante con base de goma en forma de flor que brinda mayor estabilidad, seguridad y comodidad durante el uso
+- Tamaño: 19x19x7 cm</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3224,11 +3230,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>- Material: ABS de calidad alimentaria, libre de BPA
-- • Peso Aprox.: 358 g
+          <t>- • Peso Aprox.: 358 g
 - • Capacidad - 380ml
 - • Cuchilla - Acero inoxidable 304
-- • Especificación del motor - DC 3.7V</t>
+- • Especificación del motor - DC 3.7V
+- • Tiempo de carga: 3 horas Aprox</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3253,11 +3259,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>- Material: ABS de calidad alimentaria, libre de BPA
-- • Peso Aprox.: 358 g
+          <t>- • Peso Aprox.: 358 g
 - • Capacidad - 380ml
 - • Cuchilla - Acero inoxidable 304
-- • Especificación del motor - DC 3.7V</t>
+- • Especificación del motor - DC 3.7V
+- • Tiempo de carga: 3 horas Aprox</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3282,11 +3288,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>- Material: ABS de calidad alimentaria, libre de BPA
-- • Peso Aprox.: 358 g
+          <t>- • Peso Aprox.: 358 g
 - • Capacidad - 380ml
 - • Cuchilla - Acero inoxidable 304
-- • Especificación del motor - DC 3.7V</t>
+- • Especificación del motor - DC 3.7V
+- • Tiempo de carga: 3 horas Aprox</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3311,11 +3317,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>- Material: ABS de calidad alimentaria, libre de BPA
-- • Peso Aprox.: 358 g
+          <t>- • Peso Aprox.: 358 g
 - • Capacidad - 380ml
 - • Cuchilla - Acero inoxidable 304
-- • Especificación del motor - DC 3.7V</t>
+- • Especificación del motor - DC 3.7V
+- • Tiempo de carga: 3 horas Aprox</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3369,9 +3375,7 @@
       <c r="C102" t="inlineStr">
         <is>
           <t>- Soporte impermeable para celular ideal para motociclistas y ciclistas que necesitan mantener su dispositivo visible y protegido durante el recorrido
-- Perfecto para utilizar GPS, aplicaciones de navegación o mantener el celular seguro mientras conduces
-- Características principales Diseño impermeable y resistente a salpicaduras Forro protector antigolpes Pantalla 100% táctil para usar el celular sin retirarlo Cierre hermético y seguro Instalación sencilla y firme en el manubrio Base con rotación de 360° ajustable Puede mantenerse fijo en una posición específica Brazo flexible con memoria para mejor ajuste y fijación Sistema de anclaje seguro mediante ganchos de presión Ideal para motos, bicicletas y scooters Beneficios Permite visualizar el GPS de forma segura Protege el celular contra lluvia, polvo y golpes Mantiene el dispositivo estable incluso en movimiento Fácil instalación y desmontaje Diseño práctico para uso diario y viajes Compatibilidad Compatible con la mayoría de celulares del mercado
-- Medidas aproximadas</t>
+- Perfecto para utilizar GPS, aplicaciones de navegación o mantener el celular seguro mientras conduces</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -3426,10 +3430,10 @@
       <c r="C104" t="inlineStr">
         <is>
           <t>- POTENTE ANTENA DE 36 DECIBELES PARA MEJORAR LA RECEPCIÓN DE LA SEÑAL DE LA TDT (TELEVISIÓN DIGITAL TERRESTRE)
-- CARACTERÍSTICAS DE LA ANTENA:
-- + Compatible con la TDT
 - + Conexión coaxial estándar
-- + Largo del cable 3 metros</t>
+- + Largo del cable 3 metros
+- + Material: cobre, metal, cable, imán
+- + Disfrute de la televisión digital terrestre totalmente gratis</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -3456,7 +3460,7 @@
         <is>
           <t>- 5 Recipientes comida diferentes tamaños nuevos acero inoxidable tapers bowls Cocas organizadores cocina incluye 5 tapas
 - Recipiente de acero inoxidable: Estos recipientes de almacenamiento de cocina son salsas, líquidos o sopas, debido a que la tapa cubre firmemente cada recipiente
-- preparar comidas con anticipación
+- Preparar comidas con anticipación
 - Diseño multifuncional: 5 tamaños diferentes de mixing bowl para satisfacer diversas necesidades de cocina, ahorro de espacio, no es fácil salpicar al mezclar, lo que le permite manejar fácilmente la preparación y el almacenamiento de alimentos</t>
         </is>
       </c>
@@ -3484,9 +3488,9 @@
         <is>
           <t>- Lámpara de escritorio con pinza negra, práctica y versátil para escritorios, mesas auxiliares o estanterías
 - Sistema de sujeción con pinza que permite fijarla fácilmente y optimizar el espacio de trabajo
-- Brazo flexible y cabezal ajustable para dirigir la luz según la necesidad
-- Ideal para lectura, estudio, trabajos de precisión y uso en oficina o hogar
-- Compatible con bombillos LED o incandescentes tipo E27 (según referencia)</t>
+- Compatible con bombillos LED o incandescentes tipo E27 (según referencia)
+- Funciona con voltaje amplio de 110-220V / 100-240V para mayor compatibilidad
+- Medidas aproximadas: Alto 28 cm (hasta 54-60 cm según modelo), Ancho 14 cm, Profundo 14 cm</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3514,8 +3518,8 @@
           <t>- Fabricados con materiales de alta calidad, estos ganchos son ideales para mantener tus prendas en perfecto estado
 - Aunque no son antideslizantes, su diseño triangular evita que la ropa se deslice
 - Con capacidad para varias prendas, son prácticos y funcionales para optimizar el espacio en tu armario
-- ¡No te pierdas la oportunidad de tener tus prendas organizadas con estilo!
-- Con una altura de 24 cm y un largo de 39 cm, son perfectos para colgar camisas, franelas, pantalones y shorts</t>
+- Con una altura de 24 cm y un largo de 39 cm, son perfectos para colgar camisas, franelas, pantalones y shorts
+- Este pack de 10 ganchos para ropa metálicos en color dorado es ideal para mantener tu armario organizado y con estilo</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3630,7 +3634,7 @@
           <t>- Material seguro: Esta huevera de plástico está hecha de plástico PP de alta calidad, higiénico y ecológico, libre de BPA, resistente y duradera
 - Diseño del cajón: La huevera para refrigerador tiene un diseño de cajón, a prueba de polvo y humedad, y fácil de transportar
 - Se puede acceder fácilmente a los huevos simplemente abriendo el cajón
-- su diseño hueco garantiza una buena ventilación y un efecto antimoho
+- Su diseño hueco garantiza una buena ventilación y un efecto antimoho
 - Gran capacidad: Esta huevera de gran capacidad tiene capacidad para 18-20 huevos, lo que la hace segura y no frágil</t>
         </is>
       </c>
@@ -3772,7 +3776,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>- TAPAS AJUSTABLES DE SILICONA PACK X6 UNIDADES
+          <t>- Tapas ajustables de silicona pack x6 unidades
 - Con las tapas elásticas de silicona cree un sello perfecto en cualquier recipiente de vidrio, plástico o metal, también pueden servir como reemplazo de las tapas perdidas para recipientes de forma redonda
 - Simplemente colóquelos en el lavavajillas o lávelos a mano con jabón en agua tibia después de cada uso
 - MANTENGA LOS ALIMENTOS FRESCOS: Una buena estanqueidad ayuda a mantener los alimentos frescos
@@ -3859,11 +3863,11 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>- El martillo también se utiliza para dar forma y expandir el extremo libre de remaches ligeros, remaches de cobre y remaches de fijación.Además, se ha vuelto común usar el martillo de bola para dar forma, aplanar o eliminar abolladuras en diversos metales, debido a la dureza y el peso adicionales que ofrece la herramienta
-- Las cuchillas de repuesto se encuentran dentro del cuerpo de plástico del cuchillo
+          <t>- Las cuchillas de repuesto se encuentran dentro del cuerpo de plástico del cuchillo
 - Retire la muesca negra inferior para extraer las dos cuchillas de repuesto
 - El cortador es compacto y ligero, con un agarre cómodo y cuchillas retráctiles más anchas
-- Cortador de alta resistencia, ideal para cortes más gruesos y apto para uso comercial e industrial</t>
+- Cortador de alta resistencia, ideal para cortes más gruesos y apto para uso comercial e industrial
+- Herramientas de calidad superior, robustas para tareas de fijación y reparación diarias</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3892,7 +3896,7 @@
 - Fabricada con acero al cromo vanadio arenado y cuchillas de acero al cromo molibdeno forjado
 - Medidas: Alto 24.5 cm x Ancho 9.5 cm x Largo 2.3 cm
 - Peso aproximado de 401 g, con una estructura resistente para trabajos exigentes
-- Cuchilla inferior dentada que proporciona cortes más lisos y ayuda a evitar bordes de doble marca</t>
+- Incluye 1 tijera de láminas de 250 mm, apta para trabajar con acero laminado en frío, acero inoxidable y metales no ferrosos como el aluminio</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3921,7 +3925,7 @@
 - Incluye un destornillador con mango en T que proporciona un agarre cómodo y firme, además de un mejor control al apretar y aflojar tornillos
 - Su variedad de puntas y vasos permite contar con diferentes opciones en un solo kit
 - El juego incluye 16 puntas de destornillador planas, Phillips y Torx en medidas T10, T15, T25 y T30, junto con un adaptador de 1/4", una barra de extensión y 7 llaves de vaso de 4, 5, 8, 9, 10, 11 y 12 mm
-- Sus componentes están fabricados en acero cromo vanadio, ofreciendo resistencia al desgaste y durabilidad para el uso frecuente</t>
+- Gracias a sus 24 componentes, este kit reúne diferentes herramientas para realizar tareas de fijación y ajuste de manera práctica</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -3949,8 +3953,8 @@
           <t>- Juego de brocas Steinbohrer HA597 para muro – medidas de 3 a 10 mm
 - Set de brocas para perforar muro, ladrillo, cemento, concreto y mampostería
 - Incluye diferentes medidas para trabajos de instalación, reparación y bricolaje
-- Vienen organizadas en un estuche plástico para facilitar su almacenamiento y transporte
-- Marca: Steinbohrer</t>
+- Referencia: HA597
+- Medidas: 3, 4, 5, 6, 7, 8, 9 y 10 mm</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -4008,7 +4012,7 @@
 - Su formato permite remover material de manera práctica y preparar las piezas para obtener un acabado más uniforme
 - Esta herramienta pertenece a una serie de calidad profesional y está diseñada para ofrecer un desempeño confiable durante trabajos de mantenimiento, reparación y ajuste
 - Su tamaño de 200 mm proporciona un formato cómodo para manipularla y trabajar sobre distintas piezas metálicas
-- Por su diseño, es una herramienta práctica para talleres, trabajos de bricolaje y diferentes proyectos que requieran desbastar, ajustar o pulir superficies metálicas</t>
+- Su longitud de 8 pulgadas facilita el manejo y permite realizar trabajos de acabado de manera controlada</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -4066,7 +4070,7 @@
 - Ideal para mantener el interior fresco en días calurosos
 - El soporte del ventilador es firme y seguro, no es fácil de llevar y tiene una larga vida útil
 - El diseño de doble punta de los asientos principal y co-pilo t se comparte al mismo tiempo con un alto rendimiento gracias a su conexión a cigarrera
-- Aspa de ventilador de cinco hojas, material de alta calidad</t>
+- Potencia: 8W/15W</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -4203,7 +4207,7 @@
         <is>
           <t>- Su versátil fórmula es ideal para refrescar textiles, equilibrar el aroma de tu hogar o simplemente aromatizar cualquier estancia con delicadeza
 - Presentado en un elegante frasco pino silvestre de 60 mL, es el complemento perfecto para quienes buscan bienestar y limpieza sensorial en su día a día
-- medidas: 3.5 cm x 13 cm
+- Medidas: 3.5 cm x 13 cm
 - Ideal para exhibir en estanterías o incluir en kits de regalo de tu marca
 - Es la solución técnica y sensorial que tus clientes buscan para mantener sus espacios impecables y con un aroma distintivo</t>
         </is>
@@ -4232,7 +4236,7 @@
         <is>
           <t>- Su versátil fórmula es ideal para refrescar textiles, equilibrar el aroma de tu hogar o simplemente aromatizar cualquier estancia con delicadeza
 - Presentado en un elegante frasco ámbar de 60 mL, es el complemento perfecto para quienes buscan bienestar y limpieza sensorial en su día a día
-- medidas: 3.5 cm x 13 cm
+- Medidas: 3.5 cm x 13 cm
 - Ideal para exhibir en estanterías o incluir en kits de regalo de tu marca
 - Es la solución técnica y sensorial que tus clientes buscan para mantener sus espacios impecables y con un aroma distintivo</t>
         </is>
@@ -4317,11 +4321,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>- Despierta la imaginación y la aventura de los más pequeños con el Camión Trailer de Construcción y Rescate con Sistema de Inercia! Un juguete diseñado para brindar horas de entretenimiento activo, desarrollando la motricidad fina y la creatividad en cada juego
-- Características Destacadas:
-- Acción por Inercia (Inertia Truck): ¡Solo empújalo hacia adelante y mira cómo avanza a toda velocidad sin necesidad de baterías!
-- Brazo Articulado Móvil: Cuenta con una grúa/pluma extensible y articulada, perfecta para simular rescates, obras de construcción y misiones de emergencia superdivertidas
-- Diseño Robusto y Gran Tamaño: Fabricado en plástico resistente y duradero de color rojo vibrante, equipado con ruedas todoterreno listas para superar cualquier obstáculo en casa o el parque</t>
+          <t>- Acción por Inercia (Inertia Truck): ¡Solo empújalo hacia adelante y mira cómo avanza a toda velocidad sin necesidad de baterías!
+- Detalles Realistas: Incluye estampados tipo bomberos/rescate (911) que hacen la experiencia de juego aún más inmersiva
+- Seguro y Confiable: Diseñado especialmente para niños mayores de 3 años (3+ AGES).}
+- Edad recomendada: 3 años en adelante (+3)
+- Material: Plástico ABS de alta resistencia</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -4403,11 +4407,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>- DISEÑO ERGONÓMICO
-- 16 TECLAS ADICIONALES PARA ACCESOS DIRECTOS A FUNCIONES MULTIMEDIA
+          <t>- 16 teclas adicionales para accesos directos a funciones multimedia
 - 121 TECLAS EN TOTAL
 - CONEXIÓN USB 2.0
-- LONGITUD DEL CABLE 1.19 METROS</t>
+- Longitud del cable 1.19 metros
+- Compatible con: windows, mac os 10,5 y linux</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -4436,7 +4440,7 @@
 - Su sistema de ajuste permite envolver el tobillo y regular la presión según la necesidad
 - Está fabricada con un material elástico, transpirable y suave , que se adapta al contorno del tobillo y permite mayor comodidad durante el uso
 - El cierre de velcro facilita su colocación, ajuste y retiro, además de ayudar a mantener la venda firmemente en su posición
-- Es ideal para deportistas, entrenamientos, actividades físicas y uso cotidiano , ya que ayuda a brindar estabilidad y protección al tobillo frente a movimientos que puedan generar molestias o torceduras</t>
+- El producto es de uso manual y no contiene componentes eléctricos</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -4490,8 +4494,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>- Características principales:
-- Efecto Cristal Diamante: Su estructura acrílica facetada dispersa la luz creando atractivos patrones luminosos a su alrededor
+          <t>- Efecto Cristal Diamante: Su estructura acrílica facetada dispersa la luz creando atractivos patrones luminosos a su alrededor
 - Iluminación Multicolor RGB: Combina una llama superior de tono cálido con un cuerpo transparente que proyecta cambios de luces brillantes y coloridas
 - Segura y reutilizable: Funciona sin fuego, sin cera derretida y sin humo, siendo totalmente segura para usar cerca de niños, mascotas o cortinas
 - Compacta y portátil: Alimentada por baterías (pilas de botón), ideal para colocar en mesas, repisas, altares, centro de mesa o decoración navideña sin preocuparte por cables</t>
@@ -4580,8 +4583,8 @@
           <t>- Fuerte imán y absorción, sostiene todas las herramientas pequeñas, mantiene un lugar de trabajo ordenado
 - Cubierta oxford de alta calidad, resistente al desgaste, duradera y antiincrustante
 - Malla transpirable, ligera, suave y cómoda, adecuada para 4 estaciones
-- Velcro de alta calidad, puede ajustar la longitud adecuada para su muñeca, se adapta a la mayoría de las personas
-- Costuras delicadas, costuras reforzadas, resistentes y duraderas</t>
+- Tamaño ampliado: aproximadamente 3,5 x 13.3 pulgadas
+- Material: 1680D tela de Oxford y adhesivo de nailon cinta</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -4723,10 +4726,10 @@
       <c r="C149" t="inlineStr">
         <is>
           <t>- Vaso de vino con tapa, de 12 onzas, doble pared al vacío, sin tallo, taza aislada duradera para vino, cóctel, champán, cerveza, jugo
-- Características:
 - Pueden lavarse en el lavavajillas y no se rayan como el vidrio o el plástico, simplemente enjuague y seque con un paño para eliminar las manchas de agua
 - Copa de vino de buen aislamiento: las copas de vino sin tallo con tecnología de doble pared aislada mantienen las bebidas frías durante más de 9 horas y calientes más de 5 horas
-- Más usos: este juego de copas de vino puede usarse como flauta de champán, tazas de café o vasos de agua para senderismo, picnics, autos, al aire libre, junto a la piscina, barbacoas o necesidades diarias de bebidas</t>
+- Amplia aplicación: el bonito juego de vasos es adecuado para vino, café, agua, champán, cerveza como suministros de bar o para el hogar
+- Estas copas de vino de acero inoxidable también pueden ser buenos detalles para bodas, cumpleaños o eventos</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -4780,7 +4783,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>- organizador de pastillas semanal o pastillero, diseñado para facilitar el control de la medicación o suplementos diarios
+          <t>- Organizador de pastillas semanal o pastillero, diseñado para facilitar el control de la medicación o suplementos diarios
 - Estructura: Consiste en una fila de 7 compartimentos individuales, cada uno etiquetado con los días de la semana en inglés (SUN, MON, TUE, WED, THU, FRI, SAT)
 - Diseño: El material es plástico transparente, lo que permite visualizar fácilmente el contenido sin necesidad de abrir el recipiente
 - Dimensiones: El conjunto tiene una longitud total aproximada de 13 cm y un ancho de 3 cm, lo que lo hace compacto y portátil</t>
@@ -4812,7 +4815,7 @@
 - Fabricados en PVC, un material práctico y duradero para el uso cotidiano
 - Medidas: Largo 38 cm x Ancho 38 cm x Alto 0.5 cm
 - Diseño floral que añade un detalle decorativo inspirado en elementos naturales
-- Acabado brillante que aporta una apariencia elegante y llamativa durante la presentación de la mesa</t>
+- Peso aproximado de 210 g</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -4841,7 +4844,7 @@
 - Fabricados en PVC, un material práctico y duradero para el uso cotidiano
 - Medidas: Largo 38 cm x Ancho 38 cm x Alto 0.5 cm
 - Diseño floral que añade un detalle decorativo inspirado en elementos naturales
-- Acabado brillante que aporta una apariencia elegante y llamativa durante la presentación de la mesa</t>
+- Peso aproximado de 210 g</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -4870,7 +4873,7 @@
 - Fabricados en PVC, un material práctico y duradero para el uso cotidiano
 - Medidas: Largo 38 cm x Ancho 38 cm x Alto 0.5 cm
 - Diseño floral que añade un detalle decorativo inspirado en elementos naturales
-- Acabado brillante que aporta una apariencia elegante y llamativa durante la presentación de la mesa</t>
+- Peso aproximado de 210 g</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -5069,11 +5072,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>- SOLUCIÓN IDEAL: Nuestro individual de cocina son un accesorio encantador diseñado para añadir un toque de estilo a tu hogar y proteger la mesa del comedor de las marcas de vasos y del calor de los platos
-- Fáciles de usar, prácticos y versátiles, ¡estos individuales de bambú son el elemento que le faltaba a tu casa!
+          <t>- Fáciles de usar, prácticos y versátiles, ¡estos individuales de bambú son el elemento que le faltaba a tu casa!
 - DISEÑO ECOLÓGICO: Nuestro individual para mesa de comedor está fabricado totalmente con bambú natural, un material ecológico, sostenible y de rápida regeneración que tiene un impacto ambiental muy bajo
 - ESTILO ELEGANTE Y MODERNO: Este individual de alta calidad presentan un diseño minimalista y moderno que luce genial en cualquier mesa
-- Cuentan con un trenzado de calidad y no tienen astillas</t>
+- Cuentan con un trenzado de calidad y no tienen astillas
+- PROTECCIÓN MEJORADA: Este individual ofrece un efecto aislante térmico especial que protege la mesa de posibles daños</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -5099,10 +5102,10 @@
       <c r="C162" t="inlineStr">
         <is>
           <t>- Obtén máxima iluminación y versatilidad en cualquier situación con esta Linterna Táctica LED Recargable de Alta Potencia
-- Diseñada para ofrecer un rendimiento superior en actividades al aire libre, emergencias o uso profesional, esta linterna combina un potente haz principal enfocado con un panel lateral COB de amplia cobertura
 - Su cuerpo compacto de aluminio con acabado negro mate integra un bisel táctico de impacto color naranja, ideal para situaciones de rescate o señalización
 - Además, cuenta con un indicador de carga LED circular alrededor del botón de encendido que te permite monitorear el estado de la batería en tiempo real
-- Características Principales:</t>
+- Recargable por USB: Olvídate de las baterías desechables gracias a su sistema de carga rápida y eficiente
+- Indicador de Carga: Anillo LED circular integrado en el interruptor</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -5127,11 +5130,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>- Especificaciones: Diseno de doble pared: las tazas de cafe de vidrio transparente son un diseno de doble pared, cuando las tazas de cafe de vidrio se llenan de bebidas calientes, puede proteger sus manos de quemarse, cuando las tazas se llenan de bebidas fria
-- Material principal: las tazas de cafe de vidrio de doble pared estan hechas de vidrio de borosilicato duradero, las tazas de cafe de vidrio transparente de alta calidad con material grueso, hacen que estas tazas de te transparentes resistan el uso diario, por lo que pueden contener bebidas frias y calientes
+          <t>- Material principal: las tazas de cafe de vidrio de doble pared estan hechas de vidrio de borosilicato duradero, las tazas de cafe de vidrio transparente de alta calidad con material grueso, hacen que estas tazas de te transparentes resistan el uso diario, por lo que pueden contener bebidas frias y calientes
 - Resistente y duradero, hecho de vidrio de borosilicato alto, se puede utilizar durante mucho tiempo sin preocupaciones
 - El diseño de aislamiento de doble capa es muy adecuado para bebidas frías y calientes para evitar quemaduras en las manos
-- Forma elegante, aspecto elegante, muy adecuado para beber té o café</t>
+- Forma elegante, aspecto elegante, muy adecuado para beber té o café
+- Es adecuado como cumpleaños, bodas, fiestas, día de la madre y otras situaciones</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -5160,7 +5163,7 @@
 - Luz LED suave y relajante – Emite una luz cálida y suave que crea una atmósfera relajante sin deslumbramiento, ideal para usar de noche
 - Cristal de primera calidad – Fabricada con cristal de alta claridad y sin burbujas para una transparencia y durabilidad excepcionales
 - El complemento perfecto para la decoración del hogar – Ideal para dormitorios, salas de estar, escritorios, estanterías, habitaciones infantiles o espacios de meditación
-- Regalo significativo – Un regalo único y original para cumpleaños, aniversarios, Navidad, San Valentín, graduaciones o para los amantes del espacio</t>
+- Eficiencia energética y larga duración – La luz LED de bajo consumo garantiza una larga vida útil y un uso diario seguro</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -5189,7 +5192,7 @@
 - Luz LED suave y relajante – Emite una luz cálida y suave que crea una atmósfera relajante sin deslumbramiento, ideal para usar de noche
 - Cristal de primera calidad – Fabricada con cristal de alta claridad y sin burbujas para una transparencia y durabilidad excepcionales
 - El complemento perfecto para la decoración del hogar – Ideal para dormitorios, salas de estar, escritorios, estanterías, habitaciones infantiles o espacios de meditación
-- Regalo significativo – Un regalo único y original para cumpleaños, aniversarios, Navidad, San Valentín, graduaciones o para los amantes del espacio</t>
+- Eficiencia energética y larga duración – La luz LED de bajo consumo garantiza una larga vida útil y un uso diario seguro</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -5218,7 +5221,7 @@
 - Bolsa de baño: ligera, portátil, fácil de transportar y usar, puede ofrecerte una gran comodidad
 - Bolsa malla de viaje: es adecuada para la playa, gimnasio, spa, natación, camping y deportes al aire libre, etc
 - Neceser de malla: se puede utilizar para colocar artículos de tocador, toallas, toallas de baño, cosméticos, etc
-- conveniente y práctico</t>
+- Construcción duradera: hecha de poliéster resistente, no de la tela habitual, y empleando asas de cincha con costuras cruzadas, esta bolsa de malla ofrece una solución ligera pero robusta para sus necesidades de transporte</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -5247,7 +5250,7 @@
 - Simplemente coloca nuestro soporte para gorra de béisbol donde lo necesites, dormitorios, armarios y mucho más
 - Decoración moderna: eleva tu espacio con nuestro elegante organizador de sombreros
 - Su aspecto transparente y diseño minimalista complementan varios estilos de decoración de habitaciones, lo que te permite crear una exhibición de sombreros de moda donde prefieras
-- No requiere instalación: este soporte de almacenamiento para gorra de béisbol es fácil de usar, no es necesario montarlo en una pared o puerta</t>
+- Material de alta calidad: hecho de 100% acrílico, los soportes para sombreros cuentan con una construcción transparente, lavable y robusta, asegurando un uso duradero sin preocupaciones de rotura o deformación</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -5330,11 +5333,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>- Ideal para fiestas, bodas, cumpleaños, baby showers, eventos corporativos o incluso para la decoración del hogar, este soporte es perfecto para exhibir dulces gourmet, cupcakes, minitartas, frutas, aperitivos salados o pequeños obsequios
-- Su diseño sofisticado aporta un toque de lujo a la mesa, mientras que el material acrílico de alta calidad garantiza que sea ligero, duradero y fácil de limpiar
-- Gracias a su estructura robusta y acabado en tono dorado, combina a la perfección con diversos estilos de decoración, desde el clásico hasta el moderno
+          <t>- Su diseño sofisticado aporta un toque de lujo a la mesa, mientras que el material acrílico de alta calidad garantiza que sea ligero, duradero y fácil de limpiar
 - Material: Acrílico resistente
-- Color: Transparente con detalles dorados</t>
+- Altura total: 20 cm
+- Altura hasta el segundo nivel: 13 cm
+- Diámetro de los platos: 22 cm (superior) y 26 cm (inferior)</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -5421,7 +5424,7 @@
 - Material: Plástico y Metal
 - Tamaño Producto: 13 x 10 x 3 cm / Correa extendida: 5 Metros
 - Ideal para que salgas a pasear con tu perro
-- Estira la correa hasta donde desees y presiona suavemente el botón grande, dejar presionado y soltar para que la correa se recoja automáticamente</t>
+- Gancho de metal resistente con giro de 360°</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -5448,9 +5451,9 @@
         <is>
           <t>- Material: nailon, elastano y neopreno
 - 3 niveles de temperatura de calentamiento, correspondientes a 3 colores en el controlador
-- Alivia eficazmente la artritis, el dolor en las articulaciones y la fatiga de las manos
-- La muñequera térmica ofrece calor específico para aliviar el dolor y la rigidez en tus muñecas
-- La muñequera calentada funciona con dispositivos de interfaz USB (como enchufes, computadoras y bancos de energía)</t>
+- La muñequera calentada funciona con dispositivos de interfaz USB (como enchufes, computadoras y bancos de energía)
+- Calefacción de potencia de 5 V/2 A, en interiores, se puede llevar alrededor, fácil de usar
+- Seguridad garantizada: Salto automático a temperatura media después de 5 minutos en alta temperatura</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -5477,9 +5480,9 @@
         <is>
           <t>- Diseño compacto y ligero, con peso aproximado de 63 g y distancia de funcionamiento superior a 8 m
 - Material: Plástico resistente y duradero
-- Compatibilidad: Compatible con una amplia variedad de marcas de televisores LCD, LED y HD, incluyendo LG, Samsung, Sony, Panasonic, Hisense, Kalley, Philips, RCA, Haier, Toshiba, TCL, JVC, Daewoo, Sharp, AOC, Challenger, Skyworth y otras
-- Conectividad: Tecnología infrarroja (IR) para transmitir las señales al televisor
-- Memoria: Sistema de almacenamiento de códigos que conserva la configuración al cambiar las baterías</t>
+- Compatibilidad: compatible con una amplia variedad de marcas de televisores LCD, LED y HD, incluyendo lg, samsung, sony, panasonic, hisense, kalley, philips, rca, haier, toshiba, tcl, jvc, daewoo, sharp, aoc, challenger, skyworth y otras
+- Alimentación: Funciona con 2 baterías AAA, no incluidas
+- Contenido: 1 control remoto universal</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -5508,7 +5511,7 @@
 - Diseñado para usarse dentro del lavaplatos gracias a sus partes movibles que facilitan una mejor adaptación a diferentes espacios
 - Puede colocarse también en el mueble o debajo del mesón de la cocina; su diseño de dos niveles permite aprovechar incluso los espacios más pequeños
 - Medidas específicas: altura de 37.7 cm, ancho extensible desde 50 cm hasta aproximadamente 70 cm, y largo de 26.3 cm, ideal para gabinetes estándar
-- Fabricado con plástico blanco duradero de alto impacto y tubos de acero expandibles, asegurando resistencia y larga vida útil</t>
+- Los tubos de acero se ajustan fácilmente a espacios entre 50 y 76 cm de ancho, adaptándose a la mayoría de los gabinetes de cocina o baño</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -5537,7 +5540,7 @@
 - Material: Plástico resistente al óxido
 - Capacidad de carga: hasta 20 kg (botellón de 20 litros)
 - Incluye: soporte y boquilla válvula dispensadora
-- Diseño inclinado que facilita la dispensación del agua sin necesidad de levantar el pesado botellón</t>
+- Estructura estable que soporta botellones estándar de hasta 20 litros con total seguridad</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -5565,8 +5568,8 @@
           <t>- Parlante Bluetooth portátil GTS-2422 ideal para disfrutar música en casa, exteriores y reuniones
 - Bocina de 3 pulgadas con potencia de salida de 5 W para un sonido claro y equilibrado
 - Conectividad Bluetooth compatible con dispositivos móviles, tablets y computadores
-- Incorpora puertos USB, MicroSD y radio FM para múltiples opciones de reproducción
-- Función TWS que permite enlazar dos parlantes compatibles para un sonido más amplio</t>
+- Batería interna recargable de 300 mAh con hasta 4 horas de autonomía y carga aproximada de 2 horas
+- Medidas de 11 x 8 x 14,9 cm e incluye panel frontal con botones de control integrados</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -5591,11 +5594,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>- Especificaciones:
-- Material: Plástico
-- Simulación realista: Esta flor navideña artificial tiene una apariencia delicada y una textura excelente, similar a una flor real
+          <t>- Simulación realista: Esta flor navideña artificial tiene una apariencia delicada y una textura excelente, similar a una flor real
 - Aporta un toque de color al ambiente festivo, manteniendo un brillo duradero
-- Fácil de decorar: El diseño de esta flor navideña se integra fácilmente en tu árbol de Navidad</t>
+- Fácil de decorar: El diseño de esta flor navideña se integra fácilmente en tu árbol de Navidad
+- No requiere pasos de decoración complicados for darle a tu árbol un aspecto fresco y vibrante
+- Duradera: Hecha de plástico, esta flor navideña artificial es resistente a las estaciones y al clima, manteniendo su vibrante color y hermosa forma durante mucho tiempo</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -5623,8 +5626,8 @@
           <t>- Añade un toque de sofisticación y brillo incomparable a tus espacios con nuestra Rama de Helecho Dorado de 70 cm
 - Su diseño texturizado con acabado escarchado es el complemento perfecto para elevar cualquier arreglo floral, árbol de Navidad o decoración festiva
 - Transforma tus proyectos de decoración y vitrinas comerciales esta temporada con la deslumbrante Rama de Helecho Dorado con Purpurina
-- esta pieza decorativa ha sido diseñada para capturar y reflejar la luz, creando un ambiente cálido, lujoso y sumamente elegante
-- Ya sea que estés buscando rediseñar tu árbol de Navidad, armar un centro de mesa imponente o elaborar arreglos florales profesionales para eventos y escaparates, este follaje aporta volumen, textura y un contraste sofisticado gracias a su acabado metalizado en tonos oro brillante</t>
+- Esta pieza decorativa ha sido diseñada para capturar y reflejar la luz, creando un ambiente cálido, lujoso y sumamente elegante
+- Decoración Navideña: Perfecta para sobresalir entre ramas de pino verde o nevado en el árbol de Navidad</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -5651,9 +5654,9 @@
         <is>
           <t>- Impregna tu hogar de calidez, lujo y tradición con esta rama o pick navideño decorativo con escarcha en color dorado
 - Protagonizada por una deslumbrante flor de Poinsettia con múltiples capas de pétalos recubiertos de glitter, esta pieza aporta textura, volumen y un brillo refinado a cualquier arreglo de fin de año
-- Características principales:
 - Brillo cálido y festivo: Recubrimiento total de purpurina/escarcha dorada que resalta los destellos de la luz navideña en tus espacios
-- Diseño floral de alto impacto: Incluye una flor de Nochebuena / Poinsettia de forma estructurada junto a ramas de follaje y bayas brillantes</t>
+- Diseño floral de alto impacto: Incluye una flor de Nochebuena / Poinsettia de forma estructurada junto a ramas de follaje y bayas brillantes
+- Tallo moldeable: Estructura flexible que facilita insertarla, acomodarla o fijarla fácilmente entre las ramas del árbol o en guirnaldas</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -5680,9 +5683,9 @@
         <is>
           <t>- Aporta un toque sobrio, elegante y de gran distinción a tu decoración de fin de año con esta rama o pick navideño decorativo con escarcha en color champagne
 - Diseñada con una hermosa flor de Poinsettia en la base y una espiga de follaje brillante en tonos dorados neutros, es la pieza perfecta para lograr arreglos navideños sofisticados y modernos
-- Características principales:
 - Elegante acabado champagne: Recubrimiento de purpurina/escarcha en tono oro suave que refleja la luz con destellos refinados y cálidos
-- Diseño floral integrado: Combina una flor de Nochebuena / Poinsettia, follaje de textura variada y detalles de bayas que aportan altura y volumen</t>
+- Diseño floral integrado: Combina una flor de Nochebuena / Poinsettia, follaje de textura variada y detalles de bayas que aportan altura y volumen
+- Tallo flexible y moldeable: Estructura interna de alambre ideal para entrelazar, fijar o colocar con facilidad en árboles, floreros o guirnaldas</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -5709,9 +5712,9 @@
         <is>
           <t>- Añade un toque de luz, elegancia y distinción a tu decoración navideña con esta rama o pick navideño decorativo con escarcha en color plateado
 - Con una destacada flor de Poinsettia en la base y frondosas espigas brillantes, es el elemento ideal para aportar textura y brillo a árboles de Navidad, guirnaldas y centros de mesa
-- Características principales:
 - Acabado brillante y deslumbrante: Follaje completamente cubierto de purpurina/escarcha plateada que refleja intensamente la iluminación festiva
-- Diseño floral equilibrado: Combina una flor de Nochebuena / Poinsettia, ramas de pino/helecho y detalles de bayas que suman volumen y elegancia</t>
+- Diseño floral equilibrado: Combina una flor de Nochebuena / Poinsettia, ramas de pino/helecho y detalles de bayas que suman volumen y elegancia
+- Tallo flexible y fácil de colocar: Estructura interna de alambre que permite ajustarla, doblarla o encajarla sin esfuerzo en distintas arreglos</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -5737,10 +5740,10 @@
       <c r="C184" t="inlineStr">
         <is>
           <t>- Añade delicadeza, brillo y un toque moderno a tu decoración de fin de año con esta rama o pick navideño decorativo con escarcha en color rosa
-- Diseñada con una sutil flor de Poinsettia en la base, frondosas ramas tipo helecho y un acabado reluciente, es la pieza ideal para crear combinaciones sofisticadas en árboles navideños, coronas y centros de mesa
-- Características principales:
 - Acabado brillante y romántico: Recubierta totalmente de purpurina/escarcha rosa que atrapa las luces de Navidad creando destellos suaves
-- Diseño floral integrado: Combina una flor de Nochebuena / Poinsettia con ramas texturizadas para dar altura y dimensión visual a tus arreglos</t>
+- Diseño floral integrado: Combina una flor de Nochebuena / Poinsettia con ramas texturizadas para dar altura y dimensión visual a tus arreglos
+- Tallo moldeable: Estructura de alambre flexible que facilita engancharla, trenzarla o insertarla en el árbol, guirnaldas o floreros
+- Versatilidad de decoración: Perfecta para estilos decorativos pastel, Rose Gold, románticos o temáticas de fantasía navideña</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -5766,10 +5769,10 @@
       <c r="C185" t="inlineStr">
         <is>
           <t>- Añade volumen, brillo y un toque festivo clásico a tu decoración decembrina con esta rama o pick navideño decorativo con escarcha en color rojo
-- Diseñado con una vistosa flor de Poinsettia central, ramas de follaje brillante y un tallo alargado, es el accesorio ideal para llenar de vida y luz tu árbol de Navidad, coronas, guirnaldas y arreglos florales
-- Características principales:
 - Acabado ultra brillante: Follaje y flor totalmente recubiertos de escarcha/purpurina roja que refleja la luz navideña
-- Diseño floral completo: Combina una flor de Nochebuena / Poinsettia, ramas tipo helecho/pino y detalles de bayas para mayor volumen visual</t>
+- Diseño floral completo: Combina una flor de Nochebuena / Poinsettia, ramas tipo helecho/pino y detalles de bayas para mayor volumen visual
+- Tallo moldeable y resistente: Estructura de alambre flexible que permite insertarlo, fijarlo o moldearlo fácilmente en ramas de árbol, bases de jarrones o coronas
+- Uso versátil: Perfecto para decorar árboles de Navidad, guirnaldas de chimenea o puerta, centros de mesa y arreglos florales festivos</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -5796,9 +5799,9 @@
         <is>
           <t>- Aporta frescura, elegancia y un toque nevado a tus espacios festivos con esta flor navideña decorativa de Nochebuena (Poinsettia) en color blanco
 - Sus grandes pétalos texturizados están rematados en los bordes con brillantes lentejuelas y escarcha plateada, creando un deslumbrante contraste que resalta sobre el verde del árbol
-- Características principales:
 - Detalles en lentejuelas y escarcha: Bordes de los pétalos decorados con lentejuelas plateadas que atrapan la luz y generan un brillo sofisticado
-- Tamaño destacado (30 cm): Dimensiones ideales para rellenar espacios vacíos y dar volumen a árboles, coronas y guirnaldas</t>
+- Tamaño destacado (30 cm): Dimensiones ideales para rellenar espacios vacíos y dar volumen a árboles, coronas y guirnaldas
+- Tallo flexible de 30 cm: Estructura de alambre recubierto que permite engancharla o sujetarla fácilmente en cualquier arreglo</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -5825,9 +5828,9 @@
         <is>
           <t>- Añada un toque de lujo, brillo y majestuosidad a su decoración de fin de año con esta flor navideña decorativa de Nochebuena (Poinsettia) en color dorado
 - Sus amplios pétalos combinan una textura suave acanalada con bordes delineados en lentejuelas y una capa central reluciente llena de escarcha, perfecta para hacer destacar cualquier espacio festivo
-- Características principales:
 - Bordes con lentejuelas y escarcha: Delineado de pétalos con lentejuelas doradas y centro completamente escarchado que captura la luz e intensifica el brillo
-- Tonalidad clásica y elegante: Color oro brillante tradicional, perfecto para estilos decorativos elegantes, ostentosos o de gala</t>
+- Tonalidad clásica y elegante: Color oro brillante tradicional, perfecto para estilos decorativos elegantes, ostentosos o de gala
+- Tallo flexible de alambre: Facilita la sujeción, inserción y acomodo en las ramas del árbol de Navidad, guirnaldas o coronas de entrada</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -5854,9 +5857,9 @@
         <is>
           <t>- Añada un toque cálido, sofisticado y romántico a su decoración de fin de año con esta flor navideña decorativa de Nochebuena (Poinsettia) en color Rose Gold / Palo de rosa
 - Sus delicados pétalos acolchados destacan por una combinación perfecta de texturas: bordes sutilmente delineados por lentejuelas brillantes y capas interiores completamente escarchadas que capturan la luz para realzar cualquier arreglo festivo
-- Características principales:
 - Detalle de lentejuelas y escarcha: Delineado de pétalos con lentejuelas al tono y capas centrales impregnadas de purpurina para un brillo deslumbrante
-- Tonalidad moderna y elegante: Color rosa viejo / rose gold ideal para crear paletas decorativas sofisticadas, románticas y vanguardistas</t>
+- Tonalidad moderna y elegante: Color rosa viejo / rose gold ideal para crear paletas decorativas sofisticadas, románticas y vanguardistas
+- Tallo maleable de alambre: Facilita la sujeción, enganche y acomodo en las ramas del árbol de Navidad, guirnaldas y coronas</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -5883,9 +5886,9 @@
         <is>
           <t>- Medidas: esta rama navideña tiene una altura de 70 cm y al abrir sus ramitas tiene una medida de hasta 35 cm de ancho aprox
 - La imagen muestra una rama decorativa artificial de color dorado con hojas metalizadas y pequeños frutos o perlas, ideal para arreglos navideños
-- Ideas de decoración
 - Árbol de Navidad: Coloca varias de estas ramas distribuidas en forma de abanico para dar volumen y un toque elegante
-- Centros de mesa: Combínalas con velas altas y esferas en tonos dorados o blancos dentro de un florero transparente</t>
+- Centros de mesa: Combínalas con velas altas y esferas en tonos dorados o blancos dentro de un florero transparente
+- Coronas navideñas: Úsalas como base lateral para enmarcar una corona en la puerta principal</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -5912,9 +5915,9 @@
         <is>
           <t>- Medidas: esta rama navideña tiene una altura de 70 cm y al abrir sus ramitas tiene una medida de hasta 35 cm de ancho aprox
 - La imagen muestra una rama decorativa artificial de color dorado con hojas metalizadas y pequeños frutos o perlas, ideal para arreglos navideños
-- Ideas de decoración
 - Árbol de Navidad: Coloca varias de estas ramas distribuidas en forma de abanico para dar volumen y un toque elegante
-- Centros de mesa: Combínalas con velas altas y esferas en tonos dorados o blancos dentro de un florero transparente</t>
+- Centros de mesa: Combínalas con velas altas y esferas en tonos dorados o blancos dentro de un florero transparente
+- Coronas navideñas: Úsalas como base lateral para enmarcar una corona en la puerta principal</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -5940,10 +5943,10 @@
       <c r="C191" t="inlineStr">
         <is>
           <t>- Añada ternura, calidez y un toque festivo a su hogar con este muñeco de reno navideño de peluche decorativo
-- Vestido con un detallado suéter de tejido clásico a rayas festivas, bufanda roja y encantadoras astas de fieltro, es el personaje perfecto para acompañar sus espacios durante las celebraciones de fin de año
-- Características principales:
 - Diseño detallado y tierno: Incluye suéter de punto tejido en tonos rojo, verde y blanco, bufanda acanalada y cornamenta suave en fieltro marrón
-- Textura suave y acolchada: Elaborado en materiales sintéticos de peluche de alta calidad, muy agradable al tacto y ligero de manipular</t>
+- Textura suave y acolchada: Elaborado en materiales sintéticos de peluche de alta calidad, muy agradable al tacto y ligero de manipular
+- Paleta de colores tradicional: La combinación de tonos café, rojo, verde y blanco resalta en cualquier espacio navideño
+- Versatilidad decorativa: Ideal para colocar en consolas, centros de mesa, muebles de sala, repisas o junto al árbol de Navidad</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -5969,10 +5972,10 @@
       <c r="C192" t="inlineStr">
         <is>
           <t>- Añada calidez, dulzura y encanto tradicional a su hogar con este muñeco de nieve navideño de peluche decorativo
-- Confeccionado con un detallado suéter tejido a rayas festivas, bufanda roja, faldón de encaje y gorro verde, es el personaje perfecto para llenar de vida cualquier rincón de su hogar durante las celebraciones decembrinas
-- Características principales:
 - Diseño detallado y tierno: Incluye suéter de punto tejido en tonos rojo, verde y blanco, bufanda acanalada, falda de encaje y gorro tejido a juego
-- Textura suave y acolchada: Elaborado en materiales peluche de alta calidad, muy agradable al tacto y ligero de manipular</t>
+- Textura suave y acolchada: Elaborado en materiales peluche de alta calidad, muy agradable al tacto y ligero de manipular
+- Colores navideños tradicionales: La clásica paleta en rojo, verde y blanco resalta inmediatamente en cualquier espacio
+- Versatilidad decorativa: Ideal para colocar en consolas, centros de mesa, muebles de sala, repisas o junto al árbol de Navidad</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -5998,10 +6001,10 @@
       <c r="C193" t="inlineStr">
         <is>
           <t>- Llene su hogar de espíritu festivo con este encanto de muñeco de Papá Noel navideño de peluche decorativo
-- Destacado por su vestimenta en combinación verde y roja con un divertido gorro tejido a rayas, este tierno personaje es ideal para aportar alegría y color a cualquier rincón de su hogar durante la temporada decembrina
-- Características principales:
 - Diseño exclusivo y colorido: Ataviado con un saco verde de bordes blancos, cinturón con hebilla dorada, pantalones rojos y un llamativo gorro largo tejido a rayas
-- Textura suave y liviana: Elaborado en materiales sintéticos afelpados y tejidos de excelente calidad, ligeros al tacto y fáciles de acomodar</t>
+- Textura suave y liviana: Elaborado en materiales sintéticos afelpados y tejidos de excelente calidad, ligeros al tacto y fáciles de acomodar
+- Estilo clásico y divertido: Combina elementos tradicionales de Santa Claus con un toque moderno y alegre en sus tonos
+- Versatilidad decorativa: Ideal para colocar sobre muebles, repisas, consolas, centros de mesa o recostado en el árbol de Navidad</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -6028,7 +6031,7 @@
         <is>
           <t>- Dale un toque de magia y alegría tradicional a tu hogar con este encantador Adornó Colgante de reno
 - Confeccionado con materiales suaves al tacto y un diseño detallado en relieve, este reno sosteniendo un árbol festivo es el accesorio perfecto para llenar de espíritu navideño cada rincón de tu casa
-- desde el árbol de navidad hasta la decoración de la mesa y las sillas del comedor
+- Desde el árbol de navidad hasta la decoración de la mesa y las sillas del comedor
 - Diseño Detallado y Tierno: Presenta a un clásico reno con su característica barba acolchada, su gorro texturizado y sosteniendo un hermoso pino verde de fieltro
 - Materiales Suaves y Duraderos: Elaborado con telas de alta calidad, fieltro resistente y costuras reforzadas que garantizan su durabilidad temporada tras temporada</t>
         </is>
@@ -6056,9 +6059,9 @@
       <c r="C195" t="inlineStr">
         <is>
           <t>- Dale la bienvenida a la época más mágica del año con este tierno Adorno Colgante de Papá Noel
-- DIMENSIONES: 44 CM DE ALTO 22 CM DE ANCHO
+- Dimensiones: 44 cm de alto 22 cm de ancho
 - Diseñado con detalles delicados y una combinación de tonos blancos y dorados brillantes, este accesorio es perfecto para transformar cualquier rincón de tu hogar
-- llenando tus espacios de alegría, color y el espíritu tradicional de la Navidad
+- Llenando tus espacios de alegría, color y el espíritu tradicional de la Navidad
 - Detalles Brillantes: Su gorro con líneas doradas metalizadas y un cascabel real en la punta añade un toque festivo único y un sonido sutil al mover las puertas</t>
         </is>
       </c>
@@ -6085,10 +6088,10 @@
       <c r="C196" t="inlineStr">
         <is>
           <t>- Dale la bienvenida a la época más mágica del año con este tierno Adorno Colgante de Papá Noel
-- DIMENSIONES: 44 CM DE ALTO 22 CM DE ANCHO
-- Diseñado con detalles delicados y una combinación de tonos blancos y dorados brillantes, este accesorio es perfecto para transformar cualquier rincón de tu hogar llenando tus espacios de alegría, color y el espíritu tradicional de la Navidad
+- Dimensiones: 44 cm de alto 22 cm de ancho
 - Detalles Brillantes: Su gorro con líneas doradas metalizadas y un cascabel real en la punta añade un toque festivo único y un sonido sutil al mover las puertas
-- Materiales Suaves y Duraderos: Elaborado con textiles de alta calidad que garantizan una larga vida útil, permitiéndote reutilizarlo temporada tras temporada</t>
+- Materiales Suaves y Duraderos: Elaborado con textiles de alta calidad que garantizan una larga vida útil, permitiéndote reutilizarlo temporada tras temporada
+- Fácil de Instalar: Gracias a la abertura circular integrada en la parte superior del gorro, puedes colgarlo de forma rápida y segura en manijas de puertas, pomos, ventanas o ramas del árbol de Navidad</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -6143,10 +6146,10 @@
       <c r="C198" t="inlineStr">
         <is>
           <t>- Lleve toda la alegría y tradición de las fiestas con este gorro navideño clásico de Santa Claus / Papá Noel
-- Confeccionado en una suave tela afelpada de tono rojo vivo y rematado con un suave borde de felpa blanca, es el accesorio imprescindible para lucir durante las novenas, novenas navideñas, reuniones familiares y eventos decembrinos
-- Características principales:
 - Confección suave y cómoda: Elaborado en tela aterciopelada al tacto, liviana y confortable para usar durante largos períodos
-- Medida estándar (aprox. 30 cm de base): Ajuste cómodo de talla única para adultos y jóvenes</t>
+- Medida estándar (aprox
+- 30 cm de base): Ajuste cómodo de talla única para adultos y jóvenes
+- Diseño clásico icónico: Combinación festiva en color rojo brillante con borde y pompón blanco</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -6172,10 +6175,10 @@
       <c r="C199" t="inlineStr">
         <is>
           <t>- Aporta un toque vibrante y sofisticado a tu decoración festiva con nuestra Rama de Helecho BRILLANTE de 45 cm
-- TRAE 2 HOJAS POR PAQUETE
+- Trae 2 hojas por paquete
 - Diseñada con un deslumbrante acabado escarchado, es el complemento ideal para destacar en cualquier árbol de Navidad o arreglo floral
 - Ya sea que estés redecorando tu árbol principal, diseñando centros de mesa elegantes o elaborando arreglos florales profesionales
-- este follaje escarchado refleja la luz de las guirlandas creando un ambiente cálido, moderno y sumamente acogedor</t>
+- Este follaje escarchado refleja la luz de las guirlandas creando un ambiente cálido, moderno y sumamente acogedor</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -6202,9 +6205,9 @@
         <is>
           <t>- Dale un toque especial a tu árbol de Navidad con este follaje decorativo rojo, diseñado para complementar la decoración y crear un efecto llamativo y elegante
 - Su acabado con escarcha aporta brillo y permite añadir textura y detalles a diferentes espacios del árbol
-- Gracias a su diseño con alambre, cada follaje es fácil de colocar y acomodar según el estilo que quieras lograr
 - Este kit incluye 2 unidades elaboradas en plástico, alambre y purpurina, materiales que aportan ligereza y un acabado decorativo ideal para la temporada navideña
-- Su estructura flexible facilita la colocación, el retiro y la personalización del árbol, permitiéndote distribuir las hojas de diferentes maneras</t>
+- Cada follaje tiene una altura total aproximada de 40 cm, de los cuales 20 cm corresponden únicamente al follaje, con un ancho de 13 cm y una profundidad de 1 cm
+- Cada unidad pesa aproximadamente 10 g, por lo que resulta ligera y práctica para complementar tu árbol sin recargarlo</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -6287,11 +6290,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>- Hidratación silenciosa: utilizando tecnología de , este pequeño humidificador de escritorio presenta una humidificación silenciosa para una comodidad ininterrumpida durante el trabajo el descanso, sin ninguna interrupción
-- Comodidad práctica: experimente una hidratación sin esfuerzo con este pequeño humidificador de escritorio que se adapta perfectamente a su cabecera escritorio
+          <t>- Comodidad práctica: experimente una hidratación sin esfuerzo con este pequeño humidificador de escritorio que se adapta perfectamente a su cabecera escritorio
 - Su tamaño liviano y portátil lo hacen adecuado para usar en cualquier lugar sin ocupar un espacio precioso
 - Desde viajes en coche hasta habitaciones pequeñas, disfruta de un aumento de humedad dondequiera que vayas
-- Duradero y multifuncional: elaborado por expertos con ABS+PP+silicona, este pequeño humidificador de escritorio está diseñado para durar, funciona como una relajante luz nocturna con un colorido efecto degradado y es perfecto para mejorar su espacio</t>
+- Duradero y multifuncional: elaborado por expertos con ABS+PP+silicona, este pequeño humidificador de escritorio está diseñado para durar, funciona como una relajante luz nocturna con un colorido efecto degradado y es perfecto para mejorar su espacio
+- Humidificación eficiente: disfrute de la comodidad de una niebla duradera; llénelo una vez para obtener de 6 a 12 horas de humedad continua y sin preocupaciones desde un tanque de 280 ml, lo que garantiza que su espacio l esté cómodamente humidificado</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -6316,11 +6319,11 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>- Hidratación silenciosa: utilizando tecnología de , este pequeño humidificador de escritorio presenta una humidificación silenciosa para una comodidad ininterrumpida durante el trabajo el descanso, sin ninguna interrupción
-- Comodidad práctica: experimente una hidratación sin esfuerzo con este pequeño humidificador de escritorio que se adapta perfectamente a su cabecera escritorio
+          <t>- Comodidad práctica: experimente una hidratación sin esfuerzo con este pequeño humidificador de escritorio que se adapta perfectamente a su cabecera escritorio
 - Su tamaño liviano y portátil lo hacen adecuado para usar en cualquier lugar sin ocupar un espacio precioso
 - Desde viajes en coche hasta habitaciones pequeñas, disfruta de un aumento de humedad dondequiera que vayas
-- Duradero y multifuncional: elaborado por expertos con ABS+PP+silicona, este pequeño humidificador de escritorio está diseñado para durar, funciona como una relajante luz nocturna con un colorido efecto degradado y es perfecto para mejorar su espacio</t>
+- Duradero y multifuncional: elaborado por expertos con ABS+PP+silicona, este pequeño humidificador de escritorio está diseñado para durar, funciona como una relajante luz nocturna con un colorido efecto degradado y es perfecto para mejorar su espacio
+- Humidificación eficiente: disfrute de la comodidad de una niebla duradera; llénelo una vez para obtener de 6 a 12 horas de humedad continua y sin preocupaciones desde un tanque de 280 ml, lo que garantiza que su espacio l esté cómodamente humidificado</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -6347,9 +6350,9 @@
         <is>
           <t>- Transforma el caos de tus accesorios en una exhibición digna de una joyería
 - Nuestra bandeja organizadora de terciopelo combina funcionalidad premium con un diseño minimalista que complementa cualquier espacio, desde tu tocador hasta tu vestidor
-- Diseño Versátil: Cuenta con una sección de ranuras acolchadas (ideales para anillos, pendientes o gemelos) y una sección de compartimentos abiertos (perfectos para piezas más grandes como colgantes, broches, pulseras o piedras sueltas)
 - Material: Revestimiento exterior e interior de terciopelo suave de alta calidad, diseñado para proteger las piezas delicadas de arañazos, golpes y el deslustre
-- Funcionalidad: Gracias a su perfil bajo, es ideal para organizar cajones, bandejas de tocador o para colocar dentro de joyeros más grandes</t>
+- Funcionalidad: Gracias a su perfil bajo, es ideal para organizar cajones, bandejas de tocador o para colocar dentro de joyeros más grandes
+- Además, muchos modelos de este estilo son apilables para maximizar el espacio de almacenamiento</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -6434,9 +6437,9 @@
         <is>
           <t>- Las correas son de silicona, resistentes a los arañazos y al desgaste del uso diario
 - Además, la correa de silicona es fácil de limpiar, basta con pasarla suavemente por agua para mantenerla limpia e higiénica
-- La banda de la pulsera se ha diseñado con un plegado magnético
-- Todo lo que necesitas hacer es acercar los extremos de la correa y se unirán automáticamente sin necesidad de utilizar hebillas adicionales
-- Modelo compatible: especialmente diseñado para adaptarse a los accesorios de reloj inteligente de 38mm</t>
+- Modelo compatible: especialmente diseñado para adaptarse a los accesorios de reloj inteligente de 38mm
+- Aspecto deportivo: resistente y resistente al agua
+- Además, el acero inoxidable magnético mejorado te hará ajustar la correa para adaptarse a tu muñeca fácilmente</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -6523,7 +6526,7 @@
 - Su diseño ergonómico y su mango desmontable permiten un uso cómodo y práctico, facilitando su transporte en cualquier situación, ya sea en la oficina, el gimnasio o durante actividades al aire libre
 - Fabricado con materiales de alta calidad, este termo cuenta con un interior y exterior de acero inoxidable, garantizando durabilidad y resistencia
 - La doble pared de aislamiento mantiene tus bebidas frías o calientes por más tiempo, mientras que su sistema anti-goteo asegura que no haya derrames, manteniendo tu entorno limpio y ordenado
-- Además, es libre de BPA, lo que lo convierte en una opción segura para el consumo diario</t>
+- Su superficie antideslizante proporciona un agarre firme, evitando accidentes y mejorando la experiencia de uso</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -6548,11 +6551,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>- Audífonos Bluetooth P9 Inalámbricos parámetros: 1
-- Carga USB; entrada DC 5 V 2
-- Frecuencia inalámbrica: 2.402 -2.480 GHz 4
-- Distancia inalámbrica: 10 metros 5
-- Respuesta de frecuencia: 20 Hz-20 kHz 6</t>
+          <t>- Audífonos bluetooth p9 inalámbricos parámetros: 1
+- Carga USB; entrada DC 5 v 2
+- Batería; 400 mAh 3
+- Tiempo de carga: 2 horas 9
+- El paquete incluye: 1 auricular Bluetooth,, 1 cable de carga micro USB , 1 manual de usuario</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -6577,11 +6580,10 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>- FÁCIL DE INSTALAR:
-- Puedes montarla en el parabrisas y en el salpicadero
-- OPERACIÓN CON UNA MANO:
+          <t>- Puedes montarla en el parabrisas y en el salpicadero
 - Este soporte para teléfono de coche es adecuado para bicicletas y motocicletas
-- Usted no necesita hablar ninguna herramienta, sólo tiene que desbloquear el brazo de fijación y bloquear su teléfono móvil</t>
+- Usted no necesita hablar ninguna herramienta, sólo tiene que desbloquear el brazo de fijación y bloquear su teléfono móvil
+- Se adhiere firmemente asuperficies lisas</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -6607,7 +6609,8 @@
       <c r="C214" t="inlineStr">
         <is>
           <t>- Estabilidad superior: hecho de plástico resistente al desgaste de alta calidad, este estante superior de pantalla duradero y confiable está diseñado para manejar el uso diario sin doblarse ni romperse
-- La construcción resistente mantiene tus artículos seguros y evita que se resbale o se vuelque. Perfecto para la tranquilidad y una configuración sin desorden</t>
+- La construcción resistente mantiene tus artículos seguros y evita que se resbale o se vuelque
+- Perfecto para la tranquilidad y una configuración sin desorden</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -6633,7 +6636,7 @@
       <c r="C215" t="inlineStr">
         <is>
           <t>- Tripode Plegable para un facil almacenamiento, peso ligero, tamaño compacto Compatible con Android y Iphone
-- incluye control bluetooth Cable de Carga</t>
+- Incluye control bluetooth Cable de Carga</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -6659,10 +6662,10 @@
       <c r="C216" t="inlineStr">
         <is>
           <t>- Diseñado con marcador de tiempo y citas inspiradoras, la botella para agua es perfecta para ayudarte a mantenerte motivado para beber suficiente agua durante todo el día
-- Cuenta con aspecto translúcido y escala de capacidad que te ayuda a medir tu ingesta diaria de agua fácil y claramente
-- Elección perfecta para entrenamientos, correr, senderismo, ciclismo, camping, yoga o cualquier otro deporte en casa, el gimnasio, la oficina o al aire libre
-- CARACTERÍSTICAS:
-- •Material: PC, PP, silicona</t>
+- •Material: PC, PP, silicona
+- •Pajita de silicona: tiene una pajita de silicona emergente para proteger tus dientes
+- •Incluye: Sticker 2D para cada botella
+- •Capacidad: 2000ml, 1000ml y 330ml</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -6688,10 +6691,10 @@
       <c r="C217" t="inlineStr">
         <is>
           <t>- Diseñado con marcador de tiempo y citas inspiradoras, la botella para agua es perfecta para ayudarte a mantenerte motivado para beber suficiente agua durante todo el día
-- Cuenta con aspecto translúcido y escala de capacidad que te ayuda a medir tu ingesta diaria de agua fácil y claramente
-- Elección perfecta para entrenamientos, correr, senderismo, ciclismo, camping, yoga o cualquier otro deporte en casa, el gimnasio, la oficina o al aire libre
-- CARACTERÍSTICAS:
-- •Material: PC, PP, silicona</t>
+- •Material: PC, PP, silicona
+- •Pajita de silicona: tiene una pajita de silicona emergente para proteger tus dientes
+- •Incluye: Sticker 2D para cada botella
+- •Capacidad: 2000ml, 1000ml y 330ml</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -6748,8 +6751,8 @@
           <t>- Mantén tu hidratación siempre a la mano con esta botella plegable de 600 ml, ideal para acompañarte durante actividades al aire libre, sesiones de gimnasio, rutinas de oficina y uso diario
 - Su diseño flexible permite comprimirla cuando está vacía hasta alcanzar aproximadamente 6,5 cm, facilitando su transporte y almacenamiento sin ocupar espacio innecesario
 - Está fabricada en silicona de grado alimenticio, ofreciendo una estructura práctica y resistente a impactos leves
-- Cuenta con una tapa de polipropileno, rosca hermética y tapón a presión que ayudan a mantener la bebida contenida, mientras que su diseño plegable permite utilizarla cómodamente en diferentes situaciones
-- Incluye una práctica correa de retención que facilita llevarla contigo durante tus actividades</t>
+- Incluye una práctica correa de retención que facilita llevarla contigo durante tus actividades
+- Su capacidad de 600 ml, tamaño compacto y diseño plegable la convierten en una opción funcional para quienes buscan hidratarse de manera cómoda sin cargar una botella voluminosa</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -6832,11 +6835,11 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>- Para gatos juguete eléctrico para gatos con luz LED Rollbal automático de 360 grados Juguete interactivo para gatos. Esta linda bola de juguete interactiva complacerá a tu gato
+          <t>- Para gatos juguete eléctrico para gatos con luz LED Rollbal automático de 360 grados Juguete interactivo para gatos
+- Esta linda bola de juguete interactiva complacerá a tu gato
 - Simplemente pulsa el botón y la bola comenzará automáticamente un autocarrete de 360 grados e ilumina la luz LED roja para atraer la atención de los gatos y dejar que el gato cace la pelota en la casa para divertirse y hacer ejercicio
 - Presione el interruptor para encender el juguete de pelota para gatos, encienda el modo inteligente, el juguete para gatos se apagará automáticamente después de funcionar durante 5 minutos, cambiará al modo de espera y cuando el gato toque el juguete, el juguete se despertará automáticamente
-- Con una tenue luz LED RGB, puede atraer la atención del gato
-- Modo inteligente y modo normal</t>
+- Con una tenue luz LED RGB, puede atraer la atención del gato</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
@@ -6861,11 +6864,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>- Material: neopreno
-- La superficie puede absorber instantáneamente el agua que gotea sin dejar marcas de agua o manchas
+          <t>- La superficie puede absorber instantáneamente el agua que gotea sin dejar marcas de agua o manchas
 - Antideslizante y antifugas: la alfombrilla antideslizante funciona bien en suelos lisos y húmedos
-- Fácil de limpiar y duradero: tapete de baño duradero y fácil de limpiar
-- La alfombrilla de baño permite que el agua se evapore rápidamente en el aire natural</t>
+- Dimensiones: 60 cm x 40 cm
+- Antideslizante: Equipado con una base de PVC que asegura que el tapete se mantenga firme en su lugar, incluso en superficies mojadas
+- Impermeable y de secado rápido: Evita la acumulación de humedad, protegiendo el piso y previniendo moho o malos olores</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
@@ -6890,11 +6893,11 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>- Material: neopreno
-- La superficie puede absorber instantáneamente el agua que gotea sin dejar marcas de agua o manchas
+          <t>- La superficie puede absorber instantáneamente el agua que gotea sin dejar marcas de agua o manchas
 - Antideslizante y antifugas: la alfombrilla antideslizante funciona bien en suelos lisos y húmedos
-- Fácil de limpiar y duradero: tapete de baño duradero y fácil de limpiar
-- La alfombrilla de baño permite que el agua se evapore rápidamente en el aire natural</t>
+- Dimensiones: 60 cm x 40 cm
+- Antideslizante: Equipado con una base de PVC que asegura que el tapete se mantenga firme en su lugar, incluso en superficies mojadas
+- Impermeable y de secado rápido: Evita la acumulación de humedad, protegiendo el piso y previniendo moho o malos olores</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -7038,8 +7041,8 @@
           <t>- Alivio instantáneo con extracto de ajenjo y diseño de capas duradero
 - Versátil y cómodo: diseñado para adaptarse a varias partes del cuerpo, este parche ofrece alivio rápido y transpirable
 - Ingredientes naturales con aceites de ajenjo, alcanfor, mentol y eucalipto para el máximo alivio y seguridad
-- Úsalo para dolores musculares hasta repeler mosquitos, este parche es una solución para diversas afecciones
-- Incluye: 10 parches</t>
+- Incluye: 10 parches
+- Cada empaque contiene 10 parches elaborados con extractos herbales</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -7095,9 +7098,9 @@
         <is>
           <t>- Pizarra Mágica LCD 8, 5" huntrix
 - El producto no incluye pilas
-- Con este recurso didáctico vas a potenciar el desarrollo de la creatividad mediante una superficie de escritura digital
-- Es un instrumento diseñado para facilitar la expresión artística de manera práctica y eficiente
-- Dimensiones del producto: 27x15x2 Cm</t>
+- Dimensiones del producto: 27x15x2 Cm
+- Pantalla LCD de 8, 5" para una visualización clara de los trazos
+- Fabricada en material plástico ABS de alta resistencia</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -7122,7 +7125,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>- Pizarra Mágica LCD 8, 5"
+          <t>- Pizarra mágica LCD 8, 5"
 - La imagen muestra un tablero de escritura LCD infantil con motivos de los personajes de la película Zootopia de Disney
 - Dimensiones del producto: 27x15x2 Cm
 - Pantalla: LCD sensible a la presión para dibujar y escribir sin papel
@@ -7151,11 +7154,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>- Pizarra Mágica LCD 8, 5" Toy Story
+          <t>- Pizarra mágica LCD 8, 5" toy story
 - El producto no incluye pilas
-- Con este recurso didáctico vas a potenciar el desarrollo de la creatividad mediante una superficie de escritura digital
-- Es un instrumento diseñado para facilitar la expresión artística de manera práctica y eficiente
-- Dimensiones del producto: 27x15x2 Cm</t>
+- Dimensiones del producto: 27x15x2 Cm
+- Pantalla LCD de 8, 5" para una visualización clara de los trazos
+- Fabricada en material plástico ABS de alta resistencia</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -7184,7 +7187,7 @@
 - El diseño trenzado mantiene el estilo distintivo de los cables USB de Xiaomi y suma un toque sofisticado con un patrón elegante
 - Admite carga rápida de 60W para que tus dispositivos siempre tengan energía
 - Ofrece corriente nominal de 3A para carga rápida de hasta 60W
-- Disfruta carga eficiente cuando la batería está baja</t>
+- Admite transmisión de datos a 480Mbps</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -7210,10 +7213,10 @@
       <c r="C235" t="inlineStr">
         <is>
           <t>- Organiza tus joyas con elegancia gracias a nuestro Joyero Mini Maleta Cuerina Negro
-- Características principales:
 - Medidas compactas: Con dimensiones de 17 cm * 11 cm * 6 cm, este joyero proporciona un espacio organizado sin ocupar demasiado espacio
 - Material Sintético: Fabricado con material sintético de calidad, garantizando durabilidad y resistencia para el cuidado de tus joyas
-- Mantén tus joyas ordenadas y seguras con este joyero tipo maleta. Un complemento elegante y práctico para tu colección de accesorios</t>
+- Mantén tus joyas ordenadas y seguras con este joyero tipo maleta
+- Un complemento elegante y práctico para tu colección de accesorios</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -7238,11 +7241,11 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>- Control remoto universal de reemplazo compatible con la mayoría de televisores LG
-- Modelo genérico AKB75675304, reemplazo ideal para AKB75095304, AKB75095305, AKB75095306 y AKB75095308
+          <t>- Modelo genérico AKB75675304, reemplazo ideal para AKB75095304, AKB75095305, AKB75095306 y AKB75095308
 - Botones directos para Netflix y Amazon (compatible con TVs LG 2017 en adelante)
 - Compatible con funciones Smart TV; en modelos 2016 o anteriores se accede desde la tecla Home
-- Alcance aproximado de hasta 8 metros para un control cómodo</t>
+- Alcance aproximado de hasta 8 metros para un control cómodo
+- Medidas aproximadas: 17 x 4,6 x 2 cm</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -7269,9 +7272,9 @@
         <is>
           <t>- Control remoto compatible con TV Samsung modelo BN59-01199S, diseñado para funcionar con la mayoría de televisores Samsung
 - Funcionalidad completa: permite cambiar canales, ajustar volumen, acceder a menús y modos de visualización fácilmente
-- Diseño moderno y ergonómico que se adapta cómodamente a la mano para un uso práctico y sencillo
-- Fabricado con materiales duraderos que garantizan resistencia y larga vida útil
-- Modelo del producto: BN59-01199S (Genérico)</t>
+- Modelo del producto: BN59-01199S (Genérico)
+- Alimentación mediante 2 baterías AAA (no incluidas)
+- Medidas del control: 17 x 5 cm</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -7297,10 +7300,10 @@
       <c r="C238" t="inlineStr">
         <is>
           <t>- Llena de serenidad, arte y distinción tus espacios festivos con el Farol Candelabro Decorativo ZF091
-- Este exclusivo adorno navideño de estética clásica cuenta con un acabado en tono bronce envejecido y elegantes detalles ranurados en la base y el dosel, ideales para complementar una decoración navideña sobria y refinada
 - En su panel principal exhibe una ilustración de estilo clásico de un Ángel Músico tocando el laúd en medio del cielo estrellado
 - Al encender la iluminación LED integrada, la escena proyecta una luz cálida y acogedora con delicados destellos que realzan cada detalle de la pieza
-- Características Principales:</t>
+- Iluminación Eficiente: Luz LED de tono cálido que resalta la escena celestial con un efecto brillante
+- Iluminación: Luz LED cálida con destellos de brillo</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -7326,10 +7329,10 @@
       <c r="C239" t="inlineStr">
         <is>
           <t>- Añade elegancia y calidez a tu decoración festiva con el Farol Candelabro Decorativo ZF087
-- Este adorno navideño destaca por su sofisticado diseño estilo linterna vintage en acabado bronce envejecido, complementado con sutiles grabados en relieve tanto en la base como en la cúpula
-- Su vitral frontal exhibe una encantadora escena invernal con renos/ciervos en un bosque nevado junto a una acogedora cabaña
 - Al encender la iluminación LED interior, el panel cobra vida proyectando un resplandor cálido y mágico que resalta los detalles artísticos de la ilustración
-- Características Principales: Estilo Vintage Elegante: Acabado tipo bronce antiguo con asa superior metálica para transportar o colgar fácilmente</t>
+- Iluminación Eficiente: Luz LED integrada que genera un ambiente cálido y acogedor en cualquier espacio
+- Iluminación: Luz LED cálida
+- Dimensiones: Alto: 20 cm | Ancho: 8 cm</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -7355,10 +7358,10 @@
       <c r="C240" t="inlineStr">
         <is>
           <t>- Ilumina y decora tu hogar esta Navidad con el encanto clásico del Farol Candelabro Decorativo ZF091
-- Este adorno navideño estilo farol vintage destaca por su acabado en bronce envejecido con labrados ornamentales en relieve en la base y la parte superior, aportando un toque elegante y acogedor a cualquier espacio
-- En su panel central presenta una detallada escena de la Doncella de Nieve (Snegurochka) en un vestido azul deslumbrante dentro de un paisaje invernal nevado
 - Al encenderlo, la iluminación LED cálida resalta la escena junto con destellos de purpurina, creando una atmósfera festiva y entrañable
-- Características Principales:</t>
+- Luz LED Integrada: Proporciona un brillo cálido y resalta la composición artística interior con destellos mágicos
+- Iluminación: Luz LED cálida con efecto brillante
+- Código / Referencia: ZF091</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -7384,10 +7387,10 @@
       <c r="C241" t="inlineStr">
         <is>
           <t>- Añade un toque festivo y acogedor a tus espacios con el Farol Candelabro Decorativo Navideño ZF091
-- Este adorno cuenta con un sofisticado estilo retro en acabado bronce envejecido y elegantes grabados ornamentales en relieve, ideales para resaltar la decoración de fin de año
-- En su panel frontal exhibe una encantadora ilustración de un Muñeco de Nieve con sombrero de copa, bufanda y pajaritos rojos en un paisaje invernal festivo
 - Al encender la iluminación LED integrada, la escena cobra vida con destellos brillantes y un resplandor cálido
-- Características Principales:</t>
+- Iluminación LED Cálida: Realza los detalles de la escena invernal y genera una atmósfera acogedora
+- Iluminación: Luz LED con efecto de brillo decorativo
+- Código de referencia / modelo: zf091</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -7900,7 +7903,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -7920,7 +7922,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="C6" t="inlineStr">
         <is>
@@ -7984,7 +7985,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
@@ -8009,7 +8009,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
@@ -8050,7 +8049,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>

</xml_diff>